<commit_message>
changes in IAQ for TX
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0903\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92619844-EEFB-4425-ADD6-65D075F7B6D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{707DFDA1-C8B6-4E57-960C-600B0035C3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3651,7 +3651,7 @@
     <t>YardiReviewer</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
du and llm name match css
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0908\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{707DFDA1-C8B6-4E57-960C-600B0035C3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04E24F6-4AA8-4AEC-BB6E-21E9C83A0B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3651,7 +3651,7 @@
     <t>YardiReviewer</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
changes for 3475 3474 3509 in devops
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0908\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04E24F6-4AA8-4AEC-BB6E-21E9C83A0B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAAFD610-1CDA-4E3E-A162-F624B24175F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="1204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1451" uniqueCount="1206">
   <si>
     <t>Name</t>
   </si>
@@ -3651,7 +3651,13 @@
     <t>YardiReviewer</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>ASFAExists</t>
+  </si>
+  <si>
+    <t>Affidavit of Student Financial Assistance is present in the application, manual review required.</t>
   </si>
 </sst>
 </file>
@@ -8558,7 +8564,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C524"/>
+  <dimension ref="A1:C526"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -9514,363 +9520,376 @@
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>141</v>
+        <v>1204</v>
       </c>
       <c r="B115" t="s">
-        <v>144</v>
+        <v>1205</v>
+      </c>
+      <c r="C115" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B116" t="s">
-        <v>145</v>
+        <v>144</v>
+      </c>
+      <c r="C116" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B117" t="s">
-        <v>146</v>
+        <v>145</v>
+      </c>
+      <c r="C117" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B118" t="s">
-        <v>518</v>
+        <v>146</v>
       </c>
       <c r="C118" t="s">
-        <v>596</v>
+        <v>590</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>595</v>
+        <v>139</v>
       </c>
       <c r="B119" t="s">
         <v>518</v>
       </c>
+      <c r="C119" t="s">
+        <v>596</v>
+      </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>140</v>
+        <v>595</v>
       </c>
       <c r="B120" t="s">
-        <v>123</v>
+        <v>518</v>
+      </c>
+      <c r="C120" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="B121" t="s">
-        <v>535</v>
+        <v>123</v>
+      </c>
+      <c r="C121" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B122" t="s">
-        <v>124</v>
+        <v>535</v>
+      </c>
+      <c r="C122" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>573</v>
+        <v>126</v>
       </c>
       <c r="B123" t="s">
-        <v>574</v>
+        <v>124</v>
+      </c>
+      <c r="C123" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>484</v>
+        <v>573</v>
       </c>
       <c r="B124" t="s">
-        <v>1129</v>
+        <v>574</v>
+      </c>
+      <c r="C124" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>181</v>
+        <v>484</v>
       </c>
       <c r="B126" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3">
-      <c r="A127" t="s">
-        <v>127</v>
-      </c>
-      <c r="B127" t="s">
-        <v>147</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>129</v>
+        <v>181</v>
       </c>
       <c r="B128" t="s">
-        <v>148</v>
+        <v>182</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B129" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>704</v>
+        <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>703</v>
-      </c>
-      <c r="C130" t="s">
-        <v>597</v>
+        <v>148</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B131" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>131</v>
+        <v>704</v>
       </c>
       <c r="B132" t="s">
-        <v>151</v>
+        <v>703</v>
+      </c>
+      <c r="C132" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>564</v>
+        <v>130</v>
       </c>
       <c r="B133" t="s">
-        <v>600</v>
-      </c>
-      <c r="C133" t="s">
-        <v>604</v>
+        <v>150</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>575</v>
+        <v>131</v>
       </c>
       <c r="B134" t="s">
-        <v>576</v>
+        <v>151</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>623</v>
+        <v>564</v>
       </c>
       <c r="B135" t="s">
-        <v>624</v>
+        <v>600</v>
       </c>
       <c r="C135" t="s">
-        <v>597</v>
+        <v>604</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>483</v>
+        <v>575</v>
       </c>
       <c r="B136" t="s">
-        <v>1130</v>
+        <v>576</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3">
+      <c r="A137" t="s">
+        <v>623</v>
+      </c>
+      <c r="B137" t="s">
+        <v>624</v>
+      </c>
+      <c r="C137" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
+        <v>483</v>
+      </c>
+      <c r="B138" t="s">
+        <v>1130</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3">
+      <c r="A140" t="s">
         <v>613</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B140" t="s">
         <v>614</v>
       </c>
-      <c r="C138" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3">
-      <c r="A139" t="s">
-        <v>616</v>
-      </c>
-      <c r="B139" t="s">
-        <v>1156</v>
-      </c>
-      <c r="C139" t="s">
+      <c r="C140" t="s">
         <v>615</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>153</v>
+        <v>616</v>
       </c>
       <c r="B141" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3">
-      <c r="A142" t="s">
-        <v>154</v>
-      </c>
-      <c r="B142" t="s">
-        <v>158</v>
+        <v>1156</v>
+      </c>
+      <c r="C141" t="s">
+        <v>615</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B143" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B144" t="s">
-        <v>536</v>
+        <v>158</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>500</v>
+        <v>155</v>
       </c>
       <c r="B145" t="s">
-        <v>637</v>
-      </c>
-      <c r="C145" t="s">
-        <v>638</v>
+        <v>159</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>1098</v>
+        <v>156</v>
       </c>
       <c r="B146" t="s">
-        <v>1104</v>
-      </c>
-      <c r="C146" t="s">
-        <v>597</v>
+        <v>536</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>581</v>
+        <v>500</v>
       </c>
       <c r="B147" t="s">
-        <v>582</v>
+        <v>637</v>
+      </c>
+      <c r="C147" t="s">
+        <v>638</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>482</v>
+        <v>1098</v>
       </c>
       <c r="B148" t="s">
-        <v>1157</v>
+        <v>1104</v>
+      </c>
+      <c r="C148" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3">
+      <c r="A149" t="s">
+        <v>581</v>
+      </c>
+      <c r="B149" t="s">
+        <v>582</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>185</v>
+        <v>482</v>
       </c>
       <c r="B150" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3">
-      <c r="A151" t="s">
-        <v>160</v>
-      </c>
-      <c r="B151" t="s">
-        <v>162</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>161</v>
+        <v>185</v>
       </c>
       <c r="B152" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>577</v>
+        <v>160</v>
       </c>
       <c r="B153" t="s">
-        <v>578</v>
+        <v>162</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>481</v>
+        <v>161</v>
       </c>
       <c r="B154" t="s">
-        <v>1131</v>
+        <v>163</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>625</v>
+        <v>577</v>
       </c>
       <c r="B155" t="s">
-        <v>626</v>
-      </c>
-      <c r="C155" t="s">
-        <v>597</v>
+        <v>578</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3">
+      <c r="A156" t="s">
+        <v>481</v>
+      </c>
+      <c r="B156" t="s">
+        <v>1131</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>183</v>
+        <v>625</v>
       </c>
       <c r="B157" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3">
-      <c r="A158" t="s">
-        <v>169</v>
-      </c>
-      <c r="B158" t="s">
-        <v>166</v>
-      </c>
-      <c r="C158" t="s">
-        <v>526</v>
+        <v>626</v>
+      </c>
+      <c r="C157" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="B159" t="s">
-        <v>167</v>
-      </c>
-      <c r="C159" t="s">
-        <v>526</v>
+        <v>184</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B160" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C160" t="s">
         <v>526</v>
@@ -9878,97 +9897,97 @@
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>194</v>
+        <v>164</v>
       </c>
       <c r="B161" t="s">
-        <v>193</v>
+        <v>167</v>
+      </c>
+      <c r="C161" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>191</v>
+        <v>165</v>
       </c>
       <c r="B162" t="s">
-        <v>192</v>
+        <v>168</v>
+      </c>
+      <c r="C162" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>170</v>
+        <v>194</v>
       </c>
       <c r="B163" t="s">
-        <v>171</v>
-      </c>
-      <c r="C163" t="s">
-        <v>526</v>
+        <v>193</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>579</v>
+        <v>191</v>
       </c>
       <c r="B164" t="s">
-        <v>580</v>
+        <v>192</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>470</v>
+        <v>170</v>
       </c>
       <c r="B165" t="s">
-        <v>1132</v>
+        <v>171</v>
+      </c>
+      <c r="C165" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3">
+      <c r="A166" t="s">
+        <v>579</v>
+      </c>
+      <c r="B166" t="s">
+        <v>580</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>1160</v>
+        <v>470</v>
       </c>
       <c r="B167" t="s">
-        <v>783</v>
-      </c>
-      <c r="C167" t="s">
-        <v>1161</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3">
-      <c r="A168" t="s">
-        <v>586</v>
-      </c>
-      <c r="B168" t="s">
-        <v>846</v>
-      </c>
-      <c r="C168" t="s">
-        <v>587</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>628</v>
+        <v>1160</v>
       </c>
       <c r="B169" t="s">
-        <v>629</v>
+        <v>783</v>
       </c>
       <c r="C169" t="s">
-        <v>597</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>714</v>
+        <v>586</v>
       </c>
       <c r="B170" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="C170" t="s">
-        <v>597</v>
+        <v>587</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>715</v>
+        <v>628</v>
       </c>
       <c r="B171" t="s">
-        <v>848</v>
+        <v>629</v>
       </c>
       <c r="C171" t="s">
         <v>597</v>
@@ -9976,10 +9995,10 @@
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="B172" t="s">
-        <v>700</v>
+        <v>847</v>
       </c>
       <c r="C172" t="s">
         <v>597</v>
@@ -9987,356 +10006,359 @@
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>1088</v>
+        <v>715</v>
       </c>
       <c r="B173" t="s">
-        <v>853</v>
+        <v>848</v>
       </c>
       <c r="C173" t="s">
-        <v>1089</v>
+        <v>597</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3">
+      <c r="A174" t="s">
+        <v>716</v>
+      </c>
+      <c r="B174" t="s">
+        <v>700</v>
+      </c>
+      <c r="C174" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>461</v>
+        <v>1088</v>
       </c>
       <c r="B175" t="s">
-        <v>1105</v>
-      </c>
-    </row>
-    <row r="176" spans="1:3">
-      <c r="A176" t="s">
-        <v>1111</v>
-      </c>
-      <c r="B176" t="s">
-        <v>1112</v>
-      </c>
-      <c r="C176" t="s">
-        <v>1113</v>
+        <v>853</v>
+      </c>
+      <c r="C175" t="s">
+        <v>1089</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>232</v>
+        <v>461</v>
       </c>
       <c r="B177" t="s">
-        <v>849</v>
-      </c>
-      <c r="C177" t="s">
-        <v>526</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>233</v>
+        <v>1111</v>
       </c>
       <c r="B178" t="s">
-        <v>850</v>
+        <v>1112</v>
+      </c>
+      <c r="C178" t="s">
+        <v>1113</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="B179" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="C179" t="s">
-        <v>584</v>
+        <v>526</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>685</v>
+        <v>233</v>
       </c>
       <c r="B180" t="s">
-        <v>852</v>
-      </c>
-      <c r="C180" t="s">
-        <v>597</v>
+        <v>850</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="B181" t="s">
-        <v>234</v>
+        <v>851</v>
+      </c>
+      <c r="C181" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>451</v>
+        <v>685</v>
       </c>
       <c r="B182" t="s">
-        <v>460</v>
+        <v>852</v>
+      </c>
+      <c r="C182" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B183" t="s">
-        <v>853</v>
-      </c>
-      <c r="C183" t="s">
-        <v>1090</v>
+        <v>234</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>237</v>
+        <v>451</v>
       </c>
       <c r="B184" t="s">
-        <v>854</v>
+        <v>460</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B185" t="s">
-        <v>855</v>
+        <v>853</v>
+      </c>
+      <c r="C185" t="s">
+        <v>1090</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B186" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B187" t="s">
-        <v>783</v>
+        <v>855</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>272</v>
+        <v>239</v>
       </c>
       <c r="B188" t="s">
-        <v>853</v>
-      </c>
-      <c r="C188" t="s">
-        <v>1090</v>
+        <v>856</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>299</v>
+        <v>240</v>
       </c>
       <c r="B189" t="s">
-        <v>300</v>
+        <v>783</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>589</v>
+        <v>272</v>
       </c>
       <c r="B190" t="s">
-        <v>1085</v>
+        <v>853</v>
+      </c>
+      <c r="C190" t="s">
+        <v>1090</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>606</v>
+        <v>299</v>
       </c>
       <c r="B191" t="s">
-        <v>784</v>
+        <v>300</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>671</v>
+        <v>589</v>
       </c>
       <c r="B192" t="s">
-        <v>672</v>
-      </c>
-      <c r="C192" t="s">
-        <v>597</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>684</v>
+        <v>606</v>
       </c>
       <c r="B193" t="s">
-        <v>702</v>
-      </c>
-      <c r="C193" t="s">
-        <v>597</v>
+        <v>784</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>865</v>
+        <v>671</v>
       </c>
       <c r="B194" t="s">
-        <v>866</v>
+        <v>672</v>
+      </c>
+      <c r="C194" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>469</v>
+        <v>684</v>
       </c>
       <c r="B195" t="s">
-        <v>1133</v>
+        <v>702</v>
+      </c>
+      <c r="C195" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>1185</v>
+        <v>865</v>
       </c>
       <c r="B196" t="s">
-        <v>1186</v>
+        <v>866</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3">
+      <c r="A197" t="s">
+        <v>469</v>
+      </c>
+      <c r="B197" t="s">
+        <v>1133</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>682</v>
+        <v>1185</v>
       </c>
       <c r="B198" t="s">
-        <v>683</v>
-      </c>
-      <c r="C198" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="199" spans="1:3">
-      <c r="A199" t="s">
-        <v>462</v>
-      </c>
-      <c r="B199" t="s">
-        <v>1106</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>242</v>
+        <v>682</v>
       </c>
       <c r="B200" t="s">
-        <v>857</v>
+        <v>683</v>
       </c>
       <c r="C200" t="s">
-        <v>591</v>
-      </c>
-    </row>
-    <row r="201" spans="1:3" ht="13.5" customHeight="1">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>244</v>
+        <v>462</v>
       </c>
       <c r="B201" t="s">
-        <v>858</v>
-      </c>
-      <c r="C201" t="s">
-        <v>601</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B202" t="s">
-        <v>819</v>
-      </c>
-    </row>
-    <row r="203" spans="1:3">
+        <v>857</v>
+      </c>
+      <c r="C202" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" ht="13.5" customHeight="1">
       <c r="A203" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B203" t="s">
-        <v>245</v>
+        <v>858</v>
+      </c>
+      <c r="C203" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="B204" t="s">
-        <v>248</v>
+        <v>819</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="B205" t="s">
-        <v>249</v>
-      </c>
-      <c r="C205" t="s">
-        <v>591</v>
+        <v>245</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>452</v>
+        <v>247</v>
       </c>
       <c r="B206" t="s">
-        <v>508</v>
+        <v>248</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B207" t="s">
-        <v>821</v>
+        <v>249</v>
+      </c>
+      <c r="C207" t="s">
+        <v>591</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>252</v>
+        <v>452</v>
       </c>
       <c r="B208" t="s">
-        <v>253</v>
+        <v>508</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="B209" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="B210" t="s">
-        <v>823</v>
+        <v>253</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B211" t="s">
-        <v>859</v>
-      </c>
-      <c r="C211" t="s">
-        <v>591</v>
+        <v>822</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B212" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B213" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C213" t="s">
         <v>591</v>
@@ -10344,267 +10366,267 @@
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B214" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="B215" t="s">
-        <v>270</v>
+        <v>860</v>
+      </c>
+      <c r="C215" t="s">
+        <v>591</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="B216" t="s">
-        <v>853</v>
-      </c>
-      <c r="C216" t="s">
-        <v>1090</v>
+        <v>825</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="B217" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>607</v>
+        <v>271</v>
       </c>
       <c r="B218" t="s">
-        <v>784</v>
+        <v>853</v>
+      </c>
+      <c r="C218" t="s">
+        <v>1090</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>480</v>
+        <v>273</v>
       </c>
       <c r="B219" t="s">
-        <v>1134</v>
+        <v>274</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="B220" t="s">
-        <v>603</v>
-      </c>
-      <c r="C220" t="s">
-        <v>597</v>
+        <v>784</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3">
+      <c r="A221" t="s">
+        <v>480</v>
+      </c>
+      <c r="B221" t="s">
+        <v>1134</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>463</v>
+        <v>602</v>
       </c>
       <c r="B222" t="s">
-        <v>1107</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3">
-      <c r="A223" t="s">
-        <v>453</v>
-      </c>
-      <c r="B223" t="s">
-        <v>509</v>
+        <v>603</v>
+      </c>
+      <c r="C222" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>267</v>
+        <v>463</v>
       </c>
       <c r="B224" t="s">
-        <v>785</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="225" spans="1:2">
       <c r="A225" t="s">
-        <v>268</v>
+        <v>453</v>
       </c>
       <c r="B225" t="s">
-        <v>786</v>
+        <v>509</v>
       </c>
     </row>
     <row r="226" spans="1:2">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="B226" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
     </row>
     <row r="227" spans="1:2">
       <c r="A227" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="B227" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
     </row>
     <row r="228" spans="1:2">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B228" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="229" spans="1:2">
       <c r="A229" t="s">
-        <v>608</v>
+        <v>275</v>
       </c>
       <c r="B229" t="s">
-        <v>784</v>
+        <v>789</v>
       </c>
     </row>
     <row r="230" spans="1:2">
       <c r="A230" t="s">
-        <v>479</v>
+        <v>277</v>
       </c>
       <c r="B230" t="s">
-        <v>1135</v>
+        <v>788</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" t="s">
+        <v>608</v>
+      </c>
+      <c r="B231" t="s">
+        <v>784</v>
       </c>
     </row>
     <row r="232" spans="1:2">
       <c r="A232" t="s">
-        <v>464</v>
+        <v>479</v>
       </c>
       <c r="B232" t="s">
-        <v>1108</v>
-      </c>
-    </row>
-    <row r="233" spans="1:2">
-      <c r="A233" t="s">
-        <v>454</v>
-      </c>
-      <c r="B233" t="s">
-        <v>510</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="234" spans="1:2">
       <c r="A234" t="s">
-        <v>280</v>
+        <v>464</v>
       </c>
       <c r="B234" t="s">
-        <v>778</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="235" spans="1:2">
       <c r="A235" t="s">
-        <v>281</v>
+        <v>454</v>
       </c>
       <c r="B235" t="s">
-        <v>283</v>
+        <v>510</v>
       </c>
     </row>
     <row r="236" spans="1:2">
       <c r="A236" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B236" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="237" spans="1:2">
       <c r="A237" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B237" t="s">
-        <v>781</v>
+        <v>283</v>
       </c>
     </row>
     <row r="238" spans="1:2">
       <c r="A238" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="B238" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="239" spans="1:2">
       <c r="A239" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B239" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="240" spans="1:2">
       <c r="A240" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B240" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>609</v>
+        <v>286</v>
       </c>
       <c r="B241" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>478</v>
+        <v>287</v>
       </c>
       <c r="B242" t="s">
-        <v>1136</v>
+        <v>783</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>1197</v>
+        <v>609</v>
       </c>
       <c r="B243" t="s">
-        <v>1198</v>
+        <v>784</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3">
+      <c r="A244" t="s">
+        <v>478</v>
+      </c>
+      <c r="B244" t="s">
+        <v>1136</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>465</v>
+        <v>1197</v>
       </c>
       <c r="B245" t="s">
-        <v>1109</v>
-      </c>
-    </row>
-    <row r="246" spans="1:3">
-      <c r="A246" t="s">
-        <v>449</v>
-      </c>
-      <c r="B246" t="s">
-        <v>293</v>
-      </c>
-      <c r="C246" t="s">
-        <v>526</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="B247" t="s">
-        <v>511</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>291</v>
+        <v>449</v>
       </c>
       <c r="B248" t="s">
-        <v>861</v>
+        <v>293</v>
       </c>
       <c r="C248" t="s">
         <v>526</v>
@@ -10612,306 +10634,306 @@
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>292</v>
+        <v>455</v>
       </c>
       <c r="B249" t="s">
-        <v>844</v>
+        <v>511</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>448</v>
+        <v>291</v>
       </c>
       <c r="B250" t="s">
-        <v>845</v>
+        <v>861</v>
+      </c>
+      <c r="C250" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B251" t="s">
-        <v>853</v>
-      </c>
-      <c r="C251" t="s">
-        <v>1087</v>
+        <v>844</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>295</v>
+        <v>448</v>
       </c>
       <c r="B252" t="s">
-        <v>862</v>
+        <v>845</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B253" t="s">
-        <v>863</v>
+        <v>853</v>
+      </c>
+      <c r="C253" t="s">
+        <v>1087</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B254" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B255" t="s">
-        <v>783</v>
+        <v>863</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>610</v>
+        <v>297</v>
       </c>
       <c r="B256" t="s">
-        <v>784</v>
+        <v>864</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>477</v>
+        <v>298</v>
       </c>
       <c r="B257" t="s">
-        <v>1137</v>
+        <v>783</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3">
+      <c r="A258" t="s">
+        <v>610</v>
+      </c>
+      <c r="B258" t="s">
+        <v>784</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>643</v>
+        <v>477</v>
       </c>
       <c r="B259" t="s">
-        <v>644</v>
-      </c>
-      <c r="C259" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="260" spans="1:3">
-      <c r="A260" t="s">
-        <v>494</v>
-      </c>
-      <c r="B260" t="s">
-        <v>497</v>
-      </c>
-      <c r="C260" t="s">
-        <v>524</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>495</v>
+        <v>643</v>
       </c>
       <c r="B261" t="s">
-        <v>496</v>
+        <v>644</v>
       </c>
       <c r="C261" t="s">
-        <v>525</v>
+        <v>597</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>523</v>
+        <v>494</v>
       </c>
       <c r="B262" t="s">
-        <v>537</v>
+        <v>497</v>
+      </c>
+      <c r="C262" t="s">
+        <v>524</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>315</v>
+        <v>495</v>
       </c>
       <c r="B263" t="s">
-        <v>301</v>
+        <v>496</v>
+      </c>
+      <c r="C263" t="s">
+        <v>525</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>316</v>
+        <v>523</v>
       </c>
       <c r="B264" t="s">
-        <v>302</v>
-      </c>
-      <c r="C264" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>456</v>
+        <v>315</v>
       </c>
       <c r="B265" t="s">
-        <v>512</v>
+        <v>301</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B266" t="s">
-        <v>303</v>
+        <v>302</v>
+      </c>
+      <c r="C266" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>318</v>
+        <v>456</v>
       </c>
       <c r="B267" t="s">
-        <v>304</v>
+        <v>512</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B268" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B269" t="s">
-        <v>306</v>
-      </c>
-      <c r="C269" t="s">
-        <v>526</v>
+        <v>304</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B270" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B271" t="s">
-        <v>308</v>
+        <v>306</v>
+      </c>
+      <c r="C271" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="B272" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="B273" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B274" t="s">
-        <v>311</v>
-      </c>
-      <c r="C274" t="s">
-        <v>526</v>
+        <v>309</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B275" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B276" t="s">
-        <v>313</v>
+        <v>311</v>
+      </c>
+      <c r="C276" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B277" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>476</v>
+        <v>327</v>
       </c>
       <c r="B278" t="s">
-        <v>1138</v>
+        <v>313</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3">
+      <c r="A279" t="s">
+        <v>328</v>
+      </c>
+      <c r="B279" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>541</v>
+        <v>476</v>
       </c>
       <c r="B280" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="281" spans="1:3">
-      <c r="A281" t="s">
-        <v>335</v>
-      </c>
-      <c r="B281" t="s">
-        <v>353</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>336</v>
+        <v>541</v>
       </c>
       <c r="B282" t="s">
-        <v>350</v>
+        <v>542</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B283" t="s">
-        <v>351</v>
-      </c>
-      <c r="C283" t="s">
-        <v>526</v>
+        <v>353</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>457</v>
+        <v>336</v>
       </c>
       <c r="B284" t="s">
-        <v>513</v>
+        <v>350</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>354</v>
+        <v>337</v>
       </c>
       <c r="B285" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C285" t="s">
         <v>526</v>
@@ -10919,91 +10941,88 @@
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>338</v>
+        <v>457</v>
       </c>
       <c r="B286" t="s">
-        <v>344</v>
+        <v>513</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B287" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="C287" t="s">
-        <v>503</v>
+        <v>526</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B288" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>341</v>
+        <v>355</v>
       </c>
       <c r="B289" t="s">
-        <v>347</v>
+        <v>345</v>
+      </c>
+      <c r="C289" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B290" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B291" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="B292" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>1014</v>
+        <v>342</v>
       </c>
       <c r="B293" t="s">
-        <v>1015</v>
-      </c>
-      <c r="C293" t="s">
-        <v>1010</v>
+        <v>349</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>1016</v>
+        <v>343</v>
       </c>
       <c r="B294" t="s">
-        <v>1017</v>
-      </c>
-      <c r="C294" t="s">
-        <v>1010</v>
+        <v>346</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>1018</v>
+        <v>1014</v>
       </c>
       <c r="B295" t="s">
-        <v>1019</v>
+        <v>1015</v>
       </c>
       <c r="C295" t="s">
         <v>1010</v>
@@ -11011,116 +11030,119 @@
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>475</v>
+        <v>1016</v>
       </c>
       <c r="B296" t="s">
-        <v>1139</v>
+        <v>1017</v>
+      </c>
+      <c r="C296" t="s">
+        <v>1010</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>1190</v>
+        <v>1018</v>
       </c>
       <c r="B297" t="s">
-        <v>1191</v>
+        <v>1019</v>
+      </c>
+      <c r="C297" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3">
+      <c r="A298" t="s">
+        <v>475</v>
+      </c>
+      <c r="B298" t="s">
+        <v>1139</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>645</v>
+        <v>1190</v>
       </c>
       <c r="B299" t="s">
-        <v>663</v>
-      </c>
-      <c r="C299" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="300" spans="1:3">
-      <c r="A300" t="s">
-        <v>1008</v>
-      </c>
-      <c r="B300" t="s">
-        <v>1009</v>
-      </c>
-      <c r="C300" t="s">
-        <v>1010</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>1011</v>
+        <v>645</v>
       </c>
       <c r="B301" t="s">
-        <v>1012</v>
+        <v>663</v>
       </c>
       <c r="C301" t="s">
-        <v>1010</v>
+        <v>597</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>1013</v>
+        <v>1008</v>
       </c>
       <c r="B302" t="s">
-        <v>1140</v>
+        <v>1009</v>
       </c>
       <c r="C302" t="s">
         <v>1010</v>
       </c>
     </row>
+    <row r="303" spans="1:3">
+      <c r="A303" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B303" t="s">
+        <v>1012</v>
+      </c>
+      <c r="C303" t="s">
+        <v>1010</v>
+      </c>
+    </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>641</v>
+        <v>1013</v>
       </c>
       <c r="B304" t="s">
-        <v>642</v>
+        <v>1140</v>
       </c>
       <c r="C304" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="305" spans="1:3">
-      <c r="A305" t="s">
-        <v>466</v>
-      </c>
-      <c r="B305" t="s">
-        <v>467</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>361</v>
+        <v>641</v>
       </c>
       <c r="B306" t="s">
-        <v>372</v>
+        <v>642</v>
+      </c>
+      <c r="C306" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>362</v>
+        <v>466</v>
       </c>
       <c r="B307" t="s">
-        <v>373</v>
-      </c>
-      <c r="C307" t="s">
-        <v>526</v>
+        <v>467</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>514</v>
+        <v>361</v>
       </c>
       <c r="B308" t="s">
-        <v>515</v>
+        <v>372</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B309" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C309" t="s">
         <v>526</v>
@@ -11128,155 +11150,155 @@
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>364</v>
+        <v>514</v>
       </c>
       <c r="B310" t="s">
-        <v>375</v>
-      </c>
-      <c r="C310" t="s">
-        <v>526</v>
+        <v>515</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="B311" t="s">
-        <v>527</v>
+        <v>374</v>
+      </c>
+      <c r="C311" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B312" t="s">
-        <v>376</v>
+        <v>375</v>
+      </c>
+      <c r="C312" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B313" t="s">
-        <v>377</v>
+        <v>527</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B314" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B315" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="B316" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B317" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>698</v>
+        <v>370</v>
       </c>
       <c r="B318" t="s">
-        <v>1084</v>
-      </c>
-      <c r="C318" t="s">
-        <v>597</v>
+        <v>380</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>1101</v>
+        <v>371</v>
       </c>
       <c r="B319" t="s">
-        <v>1102</v>
+        <v>381</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>473</v>
+        <v>698</v>
       </c>
       <c r="B320" t="s">
-        <v>1141</v>
+        <v>1084</v>
+      </c>
+      <c r="C320" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
-        <v>550</v>
+        <v>1101</v>
       </c>
       <c r="B321" t="s">
-        <v>551</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>1193</v>
+        <v>473</v>
       </c>
       <c r="B322" t="s">
-        <v>1194</v>
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3">
+      <c r="A323" t="s">
+        <v>550</v>
+      </c>
+      <c r="B323" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>468</v>
+        <v>1193</v>
       </c>
       <c r="B324" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="325" spans="1:3">
-      <c r="A325" t="s">
-        <v>388</v>
-      </c>
-      <c r="B325" t="s">
-        <v>399</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
-        <v>389</v>
+        <v>468</v>
       </c>
       <c r="B326" t="s">
-        <v>400</v>
-      </c>
-      <c r="C326" t="s">
-        <v>526</v>
+        <v>467</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
-        <v>458</v>
+        <v>388</v>
       </c>
       <c r="B327" t="s">
-        <v>516</v>
+        <v>399</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B328" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C328" t="s">
         <v>526</v>
@@ -11284,1448 +11306,1467 @@
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>391</v>
+        <v>458</v>
       </c>
       <c r="B329" t="s">
-        <v>402</v>
-      </c>
-      <c r="C329" t="s">
-        <v>526</v>
+        <v>516</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="B330" t="s">
-        <v>528</v>
+        <v>401</v>
+      </c>
+      <c r="C330" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B331" t="s">
-        <v>376</v>
+        <v>402</v>
+      </c>
+      <c r="C331" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B332" t="s">
-        <v>377</v>
+        <v>528</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B333" t="s">
-        <v>403</v>
+        <v>376</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="B334" t="s">
-        <v>404</v>
+        <v>377</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="B335" t="s">
-        <v>380</v>
+        <v>403</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="B336" t="s">
-        <v>381</v>
+        <v>404</v>
       </c>
     </row>
     <row r="337" spans="1:3">
       <c r="A337" t="s">
-        <v>472</v>
+        <v>397</v>
       </c>
       <c r="B337" t="s">
-        <v>1141</v>
+        <v>380</v>
       </c>
     </row>
     <row r="338" spans="1:3">
       <c r="A338" t="s">
-        <v>557</v>
+        <v>398</v>
       </c>
       <c r="B338" t="s">
-        <v>551</v>
+        <v>381</v>
       </c>
     </row>
     <row r="339" spans="1:3">
       <c r="A339" t="s">
-        <v>1195</v>
+        <v>472</v>
       </c>
       <c r="B339" t="s">
-        <v>1196</v>
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="340" spans="1:3">
+      <c r="A340" t="s">
+        <v>557</v>
+      </c>
+      <c r="B340" t="s">
+        <v>551</v>
       </c>
     </row>
     <row r="341" spans="1:3">
       <c r="A341" t="s">
-        <v>639</v>
+        <v>1195</v>
       </c>
       <c r="B341" t="s">
-        <v>640</v>
-      </c>
-      <c r="C341" t="s">
-        <v>597</v>
-      </c>
-    </row>
-    <row r="342" spans="1:3">
-      <c r="A342" t="s">
-        <v>382</v>
-      </c>
-      <c r="B342" t="s">
-        <v>558</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
-        <v>383</v>
+        <v>639</v>
       </c>
       <c r="B343" t="s">
-        <v>559</v>
+        <v>640</v>
       </c>
       <c r="C343" t="s">
-        <v>526</v>
+        <v>597</v>
       </c>
     </row>
     <row r="344" spans="1:3">
       <c r="A344" t="s">
-        <v>459</v>
+        <v>382</v>
       </c>
       <c r="B344" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B345" t="s">
-        <v>585</v>
+        <v>559</v>
+      </c>
+      <c r="C345" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>385</v>
+        <v>459</v>
       </c>
       <c r="B346" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="B347" t="s">
-        <v>562</v>
+        <v>585</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
-        <v>1118</v>
+        <v>385</v>
       </c>
       <c r="B348" t="s">
-        <v>1119</v>
-      </c>
-      <c r="C348" t="s">
-        <v>1120</v>
+        <v>561</v>
       </c>
     </row>
     <row r="349" spans="1:3">
       <c r="A349" t="s">
-        <v>471</v>
+        <v>386</v>
       </c>
       <c r="B349" t="s">
-        <v>1142</v>
+        <v>562</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3">
+      <c r="A350" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B350" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C350" t="s">
+        <v>1120</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
+        <v>471</v>
+      </c>
+      <c r="B351" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3">
+      <c r="A353" t="s">
         <v>711</v>
       </c>
-      <c r="B351" t="s">
+      <c r="B353" t="s">
         <v>712</v>
       </c>
-      <c r="C351" t="s">
+      <c r="C353" t="s">
         <v>597</v>
       </c>
     </row>
-    <row r="352" spans="1:3">
-      <c r="A352" t="s">
+    <row r="354" spans="1:3">
+      <c r="A354" t="s">
         <v>713</v>
       </c>
-      <c r="B352" t="s">
+      <c r="B354" t="s">
         <v>1143</v>
       </c>
-      <c r="C352" t="s">
+      <c r="C354" t="s">
         <v>597</v>
       </c>
     </row>
-    <row r="354" spans="1:2">
-      <c r="A354" t="s">
+    <row r="356" spans="1:3">
+      <c r="A356" t="s">
         <v>718</v>
       </c>
-      <c r="B354" t="s">
+      <c r="B356" t="s">
         <v>719</v>
       </c>
     </row>
-    <row r="355" spans="1:2">
-      <c r="A355" t="s">
+    <row r="357" spans="1:3">
+      <c r="A357" t="s">
         <v>720</v>
       </c>
-      <c r="B355" t="s">
+      <c r="B357" t="s">
         <v>721</v>
       </c>
     </row>
-    <row r="356" spans="1:2">
-      <c r="A356" t="s">
+    <row r="358" spans="1:3">
+      <c r="A358" t="s">
         <v>722</v>
       </c>
-      <c r="B356" t="s">
+      <c r="B358" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="357" spans="1:2">
-      <c r="A357" t="s">
+    <row r="359" spans="1:3">
+      <c r="A359" t="s">
         <v>724</v>
       </c>
-      <c r="B357" t="s">
+      <c r="B359" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="358" spans="1:2">
-      <c r="A358" t="s">
+    <row r="360" spans="1:3">
+      <c r="A360" t="s">
         <v>726</v>
       </c>
-      <c r="B358" t="s">
+      <c r="B360" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="359" spans="1:2">
-      <c r="A359" t="s">
+    <row r="361" spans="1:3">
+      <c r="A361" t="s">
         <v>728</v>
       </c>
-      <c r="B359" t="s">
+      <c r="B361" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="360" spans="1:2">
-      <c r="A360" t="s">
+    <row r="362" spans="1:3">
+      <c r="A362" t="s">
         <v>730</v>
       </c>
-      <c r="B360" t="s">
+      <c r="B362" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="361" spans="1:2">
-      <c r="A361" t="s">
+    <row r="363" spans="1:3">
+      <c r="A363" t="s">
         <v>732</v>
       </c>
-      <c r="B361" t="s">
+      <c r="B363" t="s">
         <v>733</v>
       </c>
     </row>
-    <row r="362" spans="1:2">
-      <c r="A362" t="s">
+    <row r="364" spans="1:3">
+      <c r="A364" t="s">
         <v>734</v>
       </c>
-      <c r="B362" t="s">
+      <c r="B364" t="s">
         <v>1180</v>
       </c>
     </row>
-    <row r="363" spans="1:2">
-      <c r="A363" t="s">
+    <row r="365" spans="1:3">
+      <c r="A365" t="s">
         <v>735</v>
       </c>
-      <c r="B363" t="s">
+      <c r="B365" t="s">
         <v>736</v>
       </c>
     </row>
-    <row r="364" spans="1:2">
-      <c r="A364" t="s">
+    <row r="366" spans="1:3">
+      <c r="A366" t="s">
         <v>737</v>
       </c>
-      <c r="B364" t="s">
+      <c r="B366" t="s">
         <v>738</v>
       </c>
     </row>
-    <row r="365" spans="1:2">
-      <c r="A365" t="s">
+    <row r="367" spans="1:3">
+      <c r="A367" t="s">
         <v>739</v>
       </c>
-      <c r="B365" t="s">
+      <c r="B367" t="s">
         <v>740</v>
       </c>
     </row>
-    <row r="366" spans="1:2">
-      <c r="A366" t="s">
+    <row r="368" spans="1:3">
+      <c r="A368" t="s">
         <v>741</v>
       </c>
-      <c r="B366" t="s">
+      <c r="B368" t="s">
         <v>742</v>
-      </c>
-    </row>
-    <row r="367" spans="1:2">
-      <c r="A367" t="s">
-        <v>743</v>
-      </c>
-      <c r="B367" t="s">
-        <v>744</v>
-      </c>
-    </row>
-    <row r="368" spans="1:2">
-      <c r="A368" t="s">
-        <v>745</v>
-      </c>
-      <c r="B368" t="s">
-        <v>746</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>747</v>
+        <v>743</v>
       </c>
       <c r="B369" t="s">
-        <v>748</v>
+        <v>744</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>1094</v>
+        <v>745</v>
       </c>
       <c r="B370" t="s">
-        <v>1095</v>
+        <v>746</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="B371" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>1117</v>
+        <v>1094</v>
       </c>
       <c r="B372" t="s">
-        <v>1144</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>1168</v>
+        <v>749</v>
       </c>
       <c r="B373" t="s">
-        <v>1169</v>
+        <v>750</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2">
+      <c r="A374" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B374" t="s">
+        <v>1144</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>751</v>
+        <v>1168</v>
       </c>
       <c r="B375" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="376" spans="1:2">
-      <c r="A376" t="s">
-        <v>753</v>
-      </c>
-      <c r="B376" t="s">
-        <v>754</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="B377" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="B378" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="B379" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="B380" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="B381" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
       <c r="B382" t="s">
-        <v>314</v>
+        <v>762</v>
       </c>
     </row>
     <row r="383" spans="1:2">
       <c r="A383" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="B383" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="B384" t="s">
-        <v>769</v>
+        <v>314</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="B385" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="B386" t="s">
-        <v>1145</v>
+        <v>769</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2">
+      <c r="A387" t="s">
+        <v>770</v>
+      </c>
+      <c r="B387" t="s">
+        <v>771</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B388" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="389" spans="1:2">
-      <c r="A389" t="s">
-        <v>774</v>
-      </c>
-      <c r="B389" t="s">
-        <v>775</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
       <c r="B390" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="B391" t="s">
-        <v>1181</v>
+        <v>775</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2">
+      <c r="A392" t="s">
+        <v>776</v>
+      </c>
+      <c r="B392" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>799</v>
+        <v>777</v>
       </c>
       <c r="B393" t="s">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="394" spans="1:2">
-      <c r="A394" t="s">
-        <v>798</v>
-      </c>
-      <c r="B394" t="s">
-        <v>797</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>792</v>
+        <v>799</v>
       </c>
       <c r="B395" t="s">
-        <v>793</v>
+        <v>800</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>790</v>
+        <v>798</v>
       </c>
       <c r="B396" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B397" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>796</v>
+        <v>790</v>
       </c>
       <c r="B398" t="s">
-        <v>1178</v>
+        <v>794</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2">
+      <c r="A399" t="s">
+        <v>791</v>
+      </c>
+      <c r="B399" t="s">
+        <v>795</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>803</v>
+        <v>796</v>
       </c>
       <c r="B400" t="s">
-        <v>808</v>
-      </c>
-    </row>
-    <row r="401" spans="1:2">
-      <c r="A401" t="s">
-        <v>810</v>
-      </c>
-      <c r="B401" t="s">
-        <v>809</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="B402" t="s">
-        <v>793</v>
+        <v>808</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>805</v>
+        <v>810</v>
       </c>
       <c r="B403" t="s">
-        <v>794</v>
+        <v>809</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="B404" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="B405" t="s">
-        <v>1146</v>
+        <v>794</v>
+      </c>
+    </row>
+    <row r="406" spans="1:2">
+      <c r="A406" t="s">
+        <v>806</v>
+      </c>
+      <c r="B406" t="s">
+        <v>795</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>815</v>
+        <v>807</v>
       </c>
       <c r="B407" t="s">
-        <v>816</v>
-      </c>
-    </row>
-    <row r="408" spans="1:2">
-      <c r="A408" t="s">
-        <v>817</v>
-      </c>
-      <c r="B408" t="s">
-        <v>1110</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="B409" t="s">
-        <v>1077</v>
+        <v>816</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="B410" t="s">
-        <v>1070</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>826</v>
+        <v>818</v>
       </c>
       <c r="B411" t="s">
-        <v>1056</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>827</v>
+        <v>820</v>
       </c>
       <c r="B412" t="s">
-        <v>1057</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="B413" t="s">
-        <v>1076</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>831</v>
+        <v>827</v>
       </c>
       <c r="B414" t="s">
-        <v>1075</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>832</v>
+        <v>828</v>
       </c>
       <c r="B415" t="s">
-        <v>1074</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="B416" t="s">
-        <v>1073</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="B417" t="s">
-        <v>1072</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="B418" t="s">
-        <v>1071</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="B419" t="s">
-        <v>825</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="B420" t="s">
-        <v>1078</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="B421" t="s">
-        <v>274</v>
+        <v>825</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="B422" t="s">
-        <v>784</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>830</v>
+        <v>838</v>
       </c>
       <c r="B423" t="s">
-        <v>603</v>
+        <v>274</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>829</v>
+        <v>839</v>
       </c>
       <c r="B424" t="s">
-        <v>1147</v>
+        <v>784</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>1192</v>
+        <v>830</v>
       </c>
       <c r="B425" t="s">
-        <v>1186</v>
+        <v>603</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>1060</v>
+        <v>829</v>
       </c>
       <c r="B426" t="s">
-        <v>1058</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>1061</v>
+        <v>1192</v>
       </c>
       <c r="B427" t="s">
-        <v>1059</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
       <c r="B428" t="s">
-        <v>1062</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>1067</v>
+        <v>1061</v>
       </c>
       <c r="B429" t="s">
-        <v>1064</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>1068</v>
+        <v>1063</v>
       </c>
       <c r="B430" t="s">
-        <v>1065</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="B431" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>1080</v>
+        <v>1068</v>
       </c>
       <c r="B432" t="s">
-        <v>1079</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>1081</v>
+        <v>1069</v>
       </c>
       <c r="B433" t="s">
-        <v>1082</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>1158</v>
+        <v>1080</v>
       </c>
       <c r="B434" t="s">
-        <v>1159</v>
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="435" spans="1:2">
+      <c r="A435" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B435" t="s">
+        <v>1082</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>899</v>
+        <v>1158</v>
       </c>
       <c r="B436" t="s">
-        <v>879</v>
-      </c>
-    </row>
-    <row r="437" spans="1:2">
-      <c r="A437" t="s">
-        <v>918</v>
-      </c>
-      <c r="B437" t="s">
-        <v>880</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>917</v>
+        <v>899</v>
       </c>
       <c r="B438" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="B439" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="B440" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
     </row>
     <row r="441" spans="1:2">
       <c r="A441" t="s">
-        <v>914</v>
+        <v>916</v>
       </c>
       <c r="B441" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>913</v>
+        <v>915</v>
       </c>
       <c r="B442" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>912</v>
+        <v>914</v>
       </c>
       <c r="B443" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>911</v>
+        <v>913</v>
       </c>
       <c r="B444" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
     </row>
     <row r="445" spans="1:2">
       <c r="A445" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="B445" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>909</v>
+        <v>911</v>
       </c>
       <c r="B446" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>919</v>
+        <v>910</v>
       </c>
       <c r="B447" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="B448" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>907</v>
+        <v>919</v>
       </c>
       <c r="B449" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="B450" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>905</v>
+        <v>907</v>
       </c>
       <c r="B451" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="B452" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="B453" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>902</v>
+        <v>904</v>
       </c>
       <c r="B454" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="B455" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
-        <v>900</v>
+        <v>902</v>
       </c>
       <c r="B456" t="s">
-        <v>1148</v>
+        <v>897</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
-        <v>1162</v>
+        <v>901</v>
       </c>
       <c r="B457" t="s">
-        <v>1163</v>
+        <v>898</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2">
+      <c r="A458" t="s">
+        <v>900</v>
+      </c>
+      <c r="B458" t="s">
+        <v>1148</v>
       </c>
     </row>
     <row r="459" spans="1:2">
       <c r="A459" t="s">
-        <v>1121</v>
+        <v>1162</v>
       </c>
       <c r="B459" t="s">
-        <v>1122</v>
-      </c>
-    </row>
-    <row r="460" spans="1:2">
-      <c r="A460" t="s">
-        <v>937</v>
-      </c>
-      <c r="B460" t="s">
-        <v>922</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
-        <v>928</v>
+        <v>1121</v>
       </c>
       <c r="B461" t="s">
-        <v>923</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>929</v>
+        <v>937</v>
       </c>
       <c r="B462" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="B463" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
       <c r="B464" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B465" t="s">
-        <v>1182</v>
+        <v>925</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="B466" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="B467" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="B468" t="s">
-        <v>1184</v>
+        <v>927</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="B469" t="s">
-        <v>1149</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1170</v>
+        <v>936</v>
       </c>
       <c r="B470" t="s">
-        <v>1171</v>
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="471" spans="1:2">
+      <c r="A471" t="s">
+        <v>935</v>
+      </c>
+      <c r="B471" t="s">
+        <v>1149</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B472" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="474" spans="1:2">
+      <c r="A474" t="s">
         <v>942</v>
       </c>
-      <c r="B472" t="s">
+      <c r="B474" t="s">
         <v>944</v>
-      </c>
-    </row>
-    <row r="473" spans="1:2">
-      <c r="A473" t="s">
-        <v>952</v>
-      </c>
-      <c r="B473" t="s">
-        <v>1150</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
+        <v>952</v>
+      </c>
+      <c r="B475" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="477" spans="1:2">
+      <c r="A477" t="s">
         <v>943</v>
       </c>
-      <c r="B475" t="s">
+      <c r="B477" t="s">
         <v>945</v>
-      </c>
-    </row>
-    <row r="476" spans="1:2">
-      <c r="A476" t="s">
-        <v>953</v>
-      </c>
-      <c r="B476" t="s">
-        <v>1151</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>950</v>
+        <v>953</v>
       </c>
       <c r="B478" t="s">
-        <v>948</v>
-      </c>
-    </row>
-    <row r="479" spans="1:2">
-      <c r="A479" t="s">
-        <v>951</v>
-      </c>
-      <c r="B479" t="s">
-        <v>949</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
-        <v>947</v>
+        <v>950</v>
       </c>
       <c r="B480" t="s">
-        <v>1152</v>
+        <v>948</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" t="s">
-        <v>1188</v>
+        <v>951</v>
       </c>
       <c r="B481" t="s">
-        <v>1189</v>
+        <v>949</v>
+      </c>
+    </row>
+    <row r="482" spans="1:2">
+      <c r="A482" t="s">
+        <v>947</v>
+      </c>
+      <c r="B482" t="s">
+        <v>1152</v>
       </c>
     </row>
     <row r="483" spans="1:2">
       <c r="A483" t="s">
-        <v>962</v>
+        <v>1188</v>
       </c>
       <c r="B483" t="s">
-        <v>955</v>
-      </c>
-    </row>
-    <row r="484" spans="1:2">
-      <c r="A484" t="s">
-        <v>963</v>
-      </c>
-      <c r="B484" t="s">
-        <v>956</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B485" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1007</v>
+        <v>963</v>
       </c>
       <c r="B486" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B487" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
     </row>
     <row r="488" spans="1:2">
       <c r="A488" t="s">
-        <v>966</v>
+        <v>1007</v>
       </c>
       <c r="B488" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
     </row>
     <row r="489" spans="1:2">
       <c r="A489" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
       <c r="B489" t="s">
-        <v>961</v>
+        <v>959</v>
+      </c>
+    </row>
+    <row r="490" spans="1:2">
+      <c r="A490" t="s">
+        <v>966</v>
+      </c>
+      <c r="B490" t="s">
+        <v>960</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>978</v>
+        <v>967</v>
       </c>
       <c r="B491" t="s">
-        <v>973</v>
-      </c>
-    </row>
-    <row r="492" spans="1:2">
-      <c r="A492" t="s">
-        <v>983</v>
-      </c>
-      <c r="B492" t="s">
-        <v>974</v>
+        <v>961</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B493" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>980</v>
+        <v>983</v>
       </c>
       <c r="B494" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
-        <v>982</v>
+        <v>979</v>
       </c>
       <c r="B495" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
     </row>
     <row r="496" spans="1:2">
       <c r="A496" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B496" t="s">
-        <v>1153</v>
+        <v>976</v>
+      </c>
+    </row>
+    <row r="497" spans="1:2">
+      <c r="A497" t="s">
+        <v>982</v>
+      </c>
+      <c r="B497" t="s">
+        <v>977</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>995</v>
+        <v>981</v>
       </c>
       <c r="B498" t="s">
-        <v>984</v>
-      </c>
-    </row>
-    <row r="499" spans="1:2">
-      <c r="A499" t="s">
-        <v>990</v>
-      </c>
-      <c r="B499" t="s">
-        <v>985</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>991</v>
+        <v>995</v>
       </c>
       <c r="B500" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="B501" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="B502" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="B503" t="s">
-        <v>1154</v>
+        <v>987</v>
+      </c>
+    </row>
+    <row r="504" spans="1:2">
+      <c r="A504" t="s">
+        <v>993</v>
+      </c>
+      <c r="B504" t="s">
+        <v>988</v>
       </c>
     </row>
     <row r="505" spans="1:2">
       <c r="A505" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
       <c r="B505" t="s">
-        <v>997</v>
-      </c>
-    </row>
-    <row r="506" spans="1:2">
-      <c r="A506" t="s">
-        <v>1002</v>
-      </c>
-      <c r="B506" t="s">
-        <v>998</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="507" spans="1:2">
       <c r="A507" t="s">
-        <v>1003</v>
+        <v>996</v>
       </c>
       <c r="B507" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
     </row>
     <row r="508" spans="1:2">
       <c r="A508" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="B508" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
     </row>
     <row r="509" spans="1:2">
       <c r="A509" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="B509" t="s">
-        <v>1001</v>
+        <v>999</v>
+      </c>
+    </row>
+    <row r="510" spans="1:2">
+      <c r="A510" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B510" t="s">
+        <v>1000</v>
       </c>
     </row>
     <row r="511" spans="1:2">
       <c r="A511" t="s">
-        <v>1028</v>
+        <v>1005</v>
       </c>
       <c r="B511" t="s">
-        <v>1029</v>
-      </c>
-    </row>
-    <row r="512" spans="1:2">
-      <c r="A512" t="s">
-        <v>1044</v>
-      </c>
-      <c r="B512" t="s">
-        <v>1030</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="513" spans="1:2">
       <c r="A513" t="s">
-        <v>1045</v>
+        <v>1028</v>
       </c>
       <c r="B513" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="514" spans="1:2">
       <c r="A514" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="B514" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="515" spans="1:2">
       <c r="A515" t="s">
-        <v>1055</v>
+        <v>1045</v>
       </c>
       <c r="B515" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="516" spans="1:2">
       <c r="A516" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B516" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="517" spans="1:2">
       <c r="A517" t="s">
-        <v>1048</v>
+        <v>1055</v>
       </c>
       <c r="B517" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="518" spans="1:2">
       <c r="A518" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="B518" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="519" spans="1:2">
       <c r="A519" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="B519" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="520" spans="1:2">
       <c r="A520" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="B520" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="521" spans="1:2">
       <c r="A521" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="B521" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="522" spans="1:2">
       <c r="A522" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="B522" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="523" spans="1:2">
       <c r="A523" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="B523" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="524" spans="1:2">
       <c r="A524" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B524" t="s">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="525" spans="1:2">
+      <c r="A525" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B525" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="526" spans="1:2">
+      <c r="A526" t="s">
         <v>1043</v>
       </c>
-      <c r="B524" t="s">
+      <c r="B526" t="s">
         <v>1042</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A478:A479 A475:A476 A460:A470 A472:A473 A481">
+  <conditionalFormatting sqref="A480:A481 A477:A478 A462:A472 A474:A475 A483">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
AS du llm match
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0909\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAAFD610-1CDA-4E3E-A162-F624B24175F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6F00E59-B860-4B6A-8912-EB4236BAFEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3651,13 +3651,13 @@
     <t>YardiReviewer</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>ASFAExists</t>
   </si>
   <si>
     <t>Affidavit of Student Financial Assistance is present in the application, manual review required.</t>
+  </si>
+  <si>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4126,7 +4126,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1203</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -9520,10 +9520,10 @@
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B115" t="s">
         <v>1204</v>
-      </c>
-      <c r="B115" t="s">
-        <v>1205</v>
       </c>
       <c r="C115" t="s">
         <v>597</v>

</xml_diff>

<commit_message>
commented out harmandeep's sequences for fuzzy matching and updated the version
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0909\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6F00E59-B860-4B6A-8912-EB4236BAFEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C5465E-39BD-478C-A5DB-1E73A4565A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21060" windowHeight="9615" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3657,7 +3657,7 @@
     <t>Affidavit of Student Financial Assistance is present in the application, manual review required.</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Library DU Model changes
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bagi.Elangovan\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C5465E-39BD-478C-A5DB-1E73A4565A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0C673D-55EF-4314-8C5F-61F4DBD74A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21060" windowHeight="9615" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3639,9 +3639,6 @@
     <t>Total Pay listed on the Work Number does not match the sum of each pay type on the Work Number.</t>
   </si>
   <si>
-    <t>DocumentTypeUserPrompt_GA.txt</t>
-  </si>
-  <si>
     <t>BackToSiteStates</t>
   </si>
   <si>
@@ -3657,7 +3654,10 @@
     <t>Affidavit of Student Financial Assistance is present in the application, manual review required.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\Bagi.Elangovan\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>DocumentTypeUserPrompt_AZ.txt</t>
   </si>
 </sst>
 </file>
@@ -4047,9 +4047,9 @@
   <dimension ref="A1:Z1005"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
-    <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
+    <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="88.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="26" width="8.7109375" customWidth="1"/>
   </cols>
@@ -4126,7 +4126,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4150,7 +4150,7 @@
         <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>1199</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
@@ -7572,26 +7572,26 @@
     </row>
     <row r="52" spans="1:2" ht="14.25" customHeight="1">
       <c r="A52" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="B52" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.25" customHeight="1">
       <c r="A53" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="B53" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="B54" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
@@ -9520,10 +9520,10 @@
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
+        <v>1202</v>
+      </c>
+      <c r="B115" t="s">
         <v>1203</v>
-      </c>
-      <c r="B115" t="s">
-        <v>1204</v>
       </c>
       <c r="C115" t="s">
         <v>597</v>

</xml_diff>

<commit_message>
3521 workflow for fuzzy matcher the employer name
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bagi.Elangovan\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0C673D-55EF-4314-8C5F-61F4DBD74A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED103809-4073-4F48-B2EB-7EFABECB4020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="4290" windowWidth="28260" windowHeight="13665" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3654,10 +3654,10 @@
     <t>Affidavit of Student Financial Assistance is present in the application, manual review required.</t>
   </si>
   <si>
-    <t>C:\Users\Bagi.Elangovan\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>DocumentTypeUserPrompt_AZ.txt</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4126,7 +4126,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4150,7 +4150,7 @@
         <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
added name matching xaml
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0914\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED103809-4073-4F48-B2EB-7EFABECB4020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{668AEF73-ACD0-4E6E-8688-54DC3EEEAB3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="28260" windowHeight="13665" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3657,7 +3657,7 @@
     <t>DocumentTypeUserPrompt_AZ.txt</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
3605 3521 updates for employer prompt
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0917\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B421EADC-F564-428C-98C6-8E766477E33E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FBE1C8F-0FB4-4E6C-90E3-D7E8AD8716E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3654,7 +3654,7 @@
     <t>Unable to validate Asset Certification of Net Family Assets. Manual review is needed. </t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
3521, bagi's findings for AZ
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0921\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C61315E-96C5-4FBD-A71C-F7E2FDBE298D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{944A3408-3D3B-406B-A065-7977F8EED28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3654,7 +3654,7 @@
     <t>Unable to validate Asset Certification of Net Family Assets. manual review required. </t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\RALUCA.ILINCA.AZUREAI-JUMP2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update rcv, hhd and csei fuzzy
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0922\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F05B601-A09D-47A3-989B-893882386427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6267AC0-4ABC-412D-8DB0-893D884D0C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3495,9 +3495,6 @@
     <t>Unable to validate Tenant Rights and Resource Guide (TRRG). Manual review is needed. </t>
   </si>
   <si>
-    <t>C:\Users\RALUCA.ILINCA.AZUREAI-JUMP2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Unable to validate Housing History Disclosure. Manual review is needed.</t>
   </si>
   <si>
@@ -3655,6 +3652,9 @@
   </si>
   <si>
     <t>Unable to validate Asset Certification of Net Family Assets. Manual review is needed. </t>
+  </si>
+  <si>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4138,7 +4138,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1150</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -8679,7 +8679,7 @@
         <v>652</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="C13" t="s">
         <v>1137</v>
@@ -8752,7 +8752,7 @@
         <v>597</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="C22" t="s">
         <v>1137</v>
@@ -8774,7 +8774,7 @@
         <v>622</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="C24" t="s">
         <v>1137</v>
@@ -8785,7 +8785,7 @@
         <v>624</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="C25" t="s">
         <v>1137</v>
@@ -8807,7 +8807,7 @@
         <v>824</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="C27" t="s">
         <v>1137</v>
@@ -8818,7 +8818,7 @@
         <v>472</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -8952,7 +8952,7 @@
         <v>487</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -9059,7 +9059,7 @@
         <v>594</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="C59" t="s">
         <v>1137</v>
@@ -9070,7 +9070,7 @@
         <v>486</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="C60" t="s">
         <v>1137</v>
@@ -9241,7 +9241,7 @@
         <v>485</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="81" spans="1:3">
@@ -9325,7 +9325,7 @@
         <v>484</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -9539,7 +9539,7 @@
         <v>483</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="115" spans="1:3">
@@ -9657,7 +9657,7 @@
         <v>482</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="127" spans="1:3">
@@ -9724,7 +9724,7 @@
         <v>561</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="C134" t="s">
         <v>1137</v>
@@ -9754,7 +9754,7 @@
         <v>481</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="139" spans="1:3">
@@ -9773,7 +9773,7 @@
         <v>608</v>
       </c>
       <c r="B140" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="C140" t="s">
         <v>607</v>
@@ -9846,7 +9846,7 @@
         <v>480</v>
       </c>
       <c r="B149" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="151" spans="1:3">
@@ -9886,7 +9886,7 @@
         <v>479</v>
       </c>
       <c r="B155" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="156" spans="1:3">
@@ -9981,7 +9981,7 @@
         <v>468</v>
       </c>
       <c r="B166" s="6" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="C166" s="6" t="s">
         <v>1141</v>
@@ -10047,7 +10047,7 @@
         <v>700</v>
       </c>
       <c r="B173" s="7" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="C173" s="2" t="s">
         <v>1137</v>
@@ -10237,7 +10237,7 @@
         <v>673</v>
       </c>
       <c r="B194" s="7" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="C194" s="2" t="s">
         <v>1137</v>
@@ -10267,7 +10267,7 @@
         <v>467</v>
       </c>
       <c r="B197" s="7" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="C197" s="2" t="s">
         <v>1137</v>
@@ -10278,7 +10278,7 @@
         <v>672</v>
       </c>
       <c r="B199" s="7" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="C199" s="2" t="s">
         <v>1137</v>
@@ -10327,7 +10327,7 @@
         <v>245</v>
       </c>
       <c r="B204" s="7" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C204" s="2" t="s">
         <v>1137</v>
@@ -10454,7 +10454,7 @@
         <v>272</v>
       </c>
       <c r="B218" s="7" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="C218" s="2" t="s">
         <v>1137</v>
@@ -10476,7 +10476,7 @@
         <v>596</v>
       </c>
       <c r="B220" s="7" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="C220" s="2" t="s">
         <v>1137</v>
@@ -10487,7 +10487,7 @@
         <v>478</v>
       </c>
       <c r="B221" s="7" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="C221" s="2" t="s">
         <v>1137</v>
@@ -10565,7 +10565,7 @@
         <v>477</v>
       </c>
       <c r="B231" s="7" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="C231" s="2" t="s">
         <v>1137</v>
@@ -10667,7 +10667,7 @@
         <v>476</v>
       </c>
       <c r="B244" s="7" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="C244" s="2" t="s">
         <v>1137</v>
@@ -10786,7 +10786,7 @@
         <v>475</v>
       </c>
       <c r="B258" s="7" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="C258" s="2" t="s">
         <v>1137</v>
@@ -10967,7 +10967,7 @@
         <v>474</v>
       </c>
       <c r="B279" s="7" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="C279" s="2" t="s">
         <v>1137</v>
@@ -11132,7 +11132,7 @@
         <v>473</v>
       </c>
       <c r="B298" s="5" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="C298" s="2" t="s">
         <v>1137</v>
@@ -11176,7 +11176,7 @@
         <v>985</v>
       </c>
       <c r="B303" s="5" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="C303" s="2" t="s">
         <v>1137</v>
@@ -11330,7 +11330,7 @@
         <v>548</v>
       </c>
       <c r="B321" s="7" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="C321" s="2" t="s">
         <v>1137</v>
@@ -11349,7 +11349,7 @@
         <v>471</v>
       </c>
       <c r="B323" s="5" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="C323" s="2" t="s">
         <v>1137</v>
@@ -11473,7 +11473,7 @@
         <v>554</v>
       </c>
       <c r="B338" s="7" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="C338" s="2" t="s">
         <v>1137</v>
@@ -11492,7 +11492,7 @@
         <v>470</v>
       </c>
       <c r="B340" s="5" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="C340" s="2" t="s">
         <v>1137</v>
@@ -11576,7 +11576,7 @@
         <v>469</v>
       </c>
       <c r="B350" s="5" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="C350" s="2" t="s">
         <v>1137</v>
@@ -11598,7 +11598,7 @@
         <v>697</v>
       </c>
       <c r="B353" s="5" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="C353" s="2" t="s">
         <v>1137</v>
@@ -11681,7 +11681,7 @@
         <v>719</v>
       </c>
       <c r="B364" s="7" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="C364" s="2" t="s">
         <v>1137</v>
@@ -11764,7 +11764,7 @@
         <v>1083</v>
       </c>
       <c r="B374" s="5" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="C374" s="2" t="s">
         <v>1137</v>
@@ -11863,7 +11863,7 @@
         <v>755</v>
       </c>
       <c r="B387" s="7" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="C387" s="2" t="s">
         <v>1137</v>
@@ -11946,7 +11946,7 @@
         <v>778</v>
       </c>
       <c r="B399" s="5" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="C399" s="2" t="s">
         <v>1137</v>
@@ -11997,7 +11997,7 @@
         <v>789</v>
       </c>
       <c r="B406" s="5" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="C406" s="2" t="s">
         <v>1137</v>
@@ -12024,7 +12024,7 @@
         <v>800</v>
       </c>
       <c r="B410" s="7" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="C410" s="2" t="s">
         <v>1137</v>
@@ -12043,7 +12043,7 @@
         <v>808</v>
       </c>
       <c r="B412" s="7" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="C412" s="2" t="s">
         <v>1137</v>
@@ -12126,7 +12126,7 @@
         <v>820</v>
       </c>
       <c r="B422" s="7" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="C422" s="2" t="s">
         <v>1137</v>
@@ -12148,7 +12148,7 @@
         <v>812</v>
       </c>
       <c r="B424" s="7" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="C424" s="2" t="s">
         <v>1137</v>
@@ -12159,7 +12159,7 @@
         <v>811</v>
       </c>
       <c r="B425" s="5" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="C425" s="2" t="s">
         <v>1137</v>
@@ -12424,7 +12424,7 @@
         <v>878</v>
       </c>
       <c r="B458" s="5" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="C458" s="2" t="s">
         <v>1137</v>
@@ -12523,7 +12523,7 @@
         <v>913</v>
       </c>
       <c r="B471" s="5" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C471" s="2" t="s">
         <v>1137</v>
@@ -12534,7 +12534,7 @@
         <v>920</v>
       </c>
       <c r="B473" s="7" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C473" s="2" t="s">
         <v>1137</v>
@@ -12545,7 +12545,7 @@
         <v>929</v>
       </c>
       <c r="B474" s="6" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="C474" s="6" t="s">
         <v>1141</v>
@@ -12567,7 +12567,7 @@
         <v>930</v>
       </c>
       <c r="B477" s="5" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="C477" s="2" t="s">
         <v>1137</v>
@@ -12602,7 +12602,7 @@
         <v>924</v>
       </c>
       <c r="B482" s="7" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="C482" s="2" t="s">
         <v>1137</v>
@@ -12613,7 +12613,7 @@
         <v>937</v>
       </c>
       <c r="B484" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="485" spans="1:3">
@@ -12661,7 +12661,7 @@
         <v>942</v>
       </c>
       <c r="B490" s="7" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="C490" s="2" t="s">
         <v>1137</v>
@@ -12809,7 +12809,7 @@
         <v>979</v>
       </c>
       <c r="B510" s="7" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="C510" s="2" t="s">
         <v>1137</v>
@@ -12924,7 +12924,7 @@
         <v>1014</v>
       </c>
       <c r="B525" s="7" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="C525" s="2" t="s">
         <v>1137</v>

</xml_diff>

<commit_message>
changes for 3548 and PL for Bagi's testing of Employer Name
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\0922\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6267AC0-4ABC-412D-8DB0-893D884D0C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868AC3E7-6D81-4507-80B5-C74D89C1523C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3654,7 +3654,7 @@
     <t>Unable to validate Asset Certification of Net Family Assets. Manual review is needed. </t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
changes in CSS.xaml for move in date and values in the LLM from DU
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76662D60-266C-45CA-84A1-9B0556D64F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA94916D-F124-4078-BD69-CB9C735082DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3621,9 +3621,6 @@
     <t>Unable to validate Asset Certification of Net Family Assets. Manual review is needed. </t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t xml:space="preserve">1040, Schedule C forms does not exist for Self-Employment Verification </t>
   </si>
   <si>
@@ -3661,6 +3658,9 @@
   </si>
   <si>
     <t>Assign button was not found in Yardi.</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4144,7 +4144,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1192</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -6174,10 +6174,10 @@
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B34" t="s">
         <v>1204</v>
-      </c>
-      <c r="B34" t="s">
-        <v>1205</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7621,10 +7621,10 @@
     </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1">
       <c r="A55" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="B55" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
@@ -10828,7 +10828,7 @@
         <v>491</v>
       </c>
       <c r="B261" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="C261" t="s">
         <v>520</v>
@@ -11534,7 +11534,7 @@
         <v>379</v>
       </c>
       <c r="B343" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="344" spans="1:3">
@@ -11542,7 +11542,7 @@
         <v>380</v>
       </c>
       <c r="B344" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="C344" t="s">
         <v>522</v>
@@ -11553,7 +11553,7 @@
         <v>456</v>
       </c>
       <c r="B345" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="346" spans="1:3">
@@ -11561,7 +11561,7 @@
         <v>381</v>
       </c>
       <c r="B346" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="347" spans="1:3">
@@ -11569,7 +11569,7 @@
         <v>382</v>
       </c>
       <c r="B347" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="348" spans="1:3">
@@ -11577,7 +11577,7 @@
         <v>383</v>
       </c>
       <c r="B348" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="349" spans="1:3">
@@ -11596,7 +11596,7 @@
         <v>468</v>
       </c>
       <c r="B350" s="5" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="C350" s="2" t="s">
         <v>1127</v>
@@ -11637,7 +11637,7 @@
         <v>696</v>
       </c>
       <c r="B356" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="357" spans="1:3">
@@ -11875,7 +11875,7 @@
         <v>744</v>
       </c>
       <c r="B386" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="387" spans="1:3">

</xml_diff>

<commit_message>
MID, EV, ACNFA update
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bagi.Elangovan\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\1001\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F0D4BEC-57F3-4A4E-9F4C-1A0EFBAB68D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FE66E4-F798-479E-85DC-FC8EBAF3014A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3660,7 +3660,7 @@
     <t>Assign button was not found in Yardi.</t>
   </si>
   <si>
-    <t>C:\Users\Bagi.Elangovan\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
changes for 3740, 3737
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\1001\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FE66E4-F798-479E-85DC-FC8EBAF3014A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F99069-74C7-4429-99EE-547FFF9C8C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11340" yWindow="240" windowWidth="13485" windowHeight="12405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3660,7 +3660,7 @@
     <t>Assign button was not found in Yardi.</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
VOE and SEC fixes
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\1007\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F99069-74C7-4429-99EE-547FFF9C8C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F0EA44B-A0E5-476C-9605-AD96821BA98D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11340" yWindow="240" windowWidth="13485" windowHeight="12405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="735" windowWidth="21495" windowHeight="10875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3660,7 +3660,7 @@
     <t>Assign button was not found in Yardi.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
EV - TX and EV - GA parallel processing
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110B3355-9D8B-4D98-B571-8856FE6767A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785766A1-5F66-428F-9302-D4366F4EEFE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3660,13 +3660,13 @@
     <t>Assign button was not found in Yardi.</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>DelayAfterTime</t>
   </si>
   <si>
     <t>ElementTimeout</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4150,7 +4150,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1205</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7579,18 +7579,18 @@
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
       <c r="A49" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="B49" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1">
       <c r="A50" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="B50" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
Update icw income type fuzzy match
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\1014\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785766A1-5F66-428F-9302-D4366F4EEFE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8174209E-61A1-4FE0-9BD8-B90486D56657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3666,7 +3666,7 @@
     <t>ElementTimeout</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
changes for ICW Income Type amnd EV Model
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\1014\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8174209E-61A1-4FE0-9BD8-B90486D56657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99576DFB-D16C-4633-80D3-E36A412B827D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="28260" windowHeight="13665" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1510" uniqueCount="1208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="1209">
   <si>
     <t>Name</t>
   </si>
@@ -3666,14 +3666,17 @@
     <t>ElementTimeout</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>UnsupportedIncomeTypesFilePath</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -3703,6 +3706,11 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -3730,7 +3738,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3743,6 +3751,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7649,7 +7658,14 @@
         <v>1202</v>
       </c>
     </row>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="58" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A58" s="8" t="s">
+        <v>1208</v>
+      </c>
+      <c r="B58" s="8" t="s">
+        <v>1208</v>
+      </c>
+    </row>
     <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="61" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
changes for 3792, 3870, 3848
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bagi.Elangovan\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E19FC9AC-3E1E-4DB1-91B5-C46E93573A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D916EA8C-F29D-4B87-9B78-FCAB61CD2C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="16740" windowHeight="8250" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1512" uniqueCount="1209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="1210">
   <si>
     <t>Name</t>
   </si>
@@ -3669,7 +3669,10 @@
     <t>UnsupportedIncomeTypesFilePath</t>
   </si>
   <si>
-    <t>C:\Users\Bagi.Elangovan\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>TX_VSAVerificationProperties</t>
   </si>
 </sst>
 </file>
@@ -7666,7 +7669,14 @@
         <v>1207</v>
       </c>
     </row>
-    <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="59" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A59" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1209</v>
+      </c>
+    </row>
     <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="62" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
updated the config file with the newest assets
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D916EA8C-F29D-4B87-9B78-FCAB61CD2C6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F0857E-F12D-4A46-AE7D-A85A54D746FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="16740" windowHeight="8250" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1514" uniqueCount="1210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1516" uniqueCount="1211">
   <si>
     <t>Name</t>
   </si>
@@ -3673,13 +3673,16 @@
   </si>
   <si>
     <t>TX_VSAVerificationProperties</t>
+  </si>
+  <si>
+    <t>TX_NoAssetsCheckProperties</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -3710,8 +3713,15 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Segoe UI"/>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -3741,7 +3751,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3755,6 +3765,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7171,23 +7182,23 @@
   <dimension ref="A1:Z1017"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="2" width="37.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="50.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="26" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E1" s="1"/>
@@ -7214,84 +7225,104 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>684</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>684</v>
       </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>45</v>
       </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>48</v>
       </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>49</v>
       </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>50</v>
       </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>51</v>
       </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>52</v>
       </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>54</v>
       </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
@@ -7300,388 +7331,493 @@
       <c r="B12" s="2" t="s">
         <v>205</v>
       </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>500</v>
       </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" t="s">
+      <c r="A14" s="2" t="s">
         <v>501</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>501</v>
       </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A15" t="s">
+      <c r="A15" s="2" t="s">
         <v>502</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>502</v>
       </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>503</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>503</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A17" t="s">
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A17" s="2" t="s">
         <v>540</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>540</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A18" t="s">
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A18" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>542</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A19" t="s">
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A19" s="2" t="s">
         <v>544</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>544</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A20" t="s">
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A20" s="2" t="s">
         <v>541</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="2" t="s">
         <v>541</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A21" t="s">
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A21" s="2" t="s">
         <v>543</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="2" t="s">
         <v>543</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A22" t="s">
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A22" s="2" t="s">
         <v>1072</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="2" t="s">
         <v>1072</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A23" t="s">
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A23" s="2" t="s">
         <v>553</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="2" t="s">
         <v>553</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A24" t="s">
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A24" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A25" t="s">
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+    </row>
+    <row r="25" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A25" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" ht="14.25" customHeight="1">
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" spans="1:4" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="2" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" ht="14.25" customHeight="1">
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+    </row>
+    <row r="27" spans="1:4" ht="14.25" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>230</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" ht="14.25" customHeight="1">
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+    </row>
+    <row r="28" spans="1:4" ht="14.25" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>254</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A29" t="s">
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+    </row>
+    <row r="29" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A29" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="2" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A30" t="s">
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A30" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="2" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A31" t="s">
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A31" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="2" t="s">
         <v>439</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A32" t="s">
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A32" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="2" t="s">
         <v>440</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" ht="14.25" customHeight="1">
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="1:4" ht="14.25" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>515</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>515</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A34" t="s">
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A34" s="2" t="s">
         <v>517</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="2" t="s">
         <v>517</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" ht="14.25" customHeight="1">
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+    </row>
+    <row r="35" spans="1:4" ht="14.25" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="2" t="s">
         <v>516</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A36" t="s">
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+    </row>
+    <row r="36" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A36" s="2" t="s">
         <v>518</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="2" t="s">
         <v>518</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A37" t="s">
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A37" s="2" t="s">
         <v>534</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="2" t="s">
         <v>534</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A38" t="s">
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A38" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="2" t="s">
         <v>535</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A39" t="s">
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+    </row>
+    <row r="39" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A39" s="2" t="s">
         <v>573</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="2" t="s">
         <v>573</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A40" t="s">
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A40" s="2" t="s">
         <v>1108</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="2" t="s">
         <v>1108</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A41" t="s">
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A41" s="2" t="s">
         <v>655</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="2" t="s">
         <v>655</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A42" t="s">
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A42" s="2" t="s">
         <v>582</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="2" t="s">
         <v>582</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A43" t="s">
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A43" s="2" t="s">
         <v>615</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="2" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A44" t="s">
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A44" s="2" t="s">
         <v>619</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="2" t="s">
         <v>619</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A45" t="s">
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+    </row>
+    <row r="45" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A45" s="2" t="s">
         <v>662</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="2" t="s">
         <v>662</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A46" t="s">
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+    </row>
+    <row r="46" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A46" s="2" t="s">
         <v>984</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="2" t="s">
         <v>984</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A47" t="s">
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+    </row>
+    <row r="47" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A47" s="2" t="s">
         <v>985</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="2" t="s">
         <v>985</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A48" t="s">
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+    </row>
+    <row r="48" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A48" s="2" t="s">
         <v>986</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="2" t="s">
         <v>986</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A49" t="s">
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+    </row>
+    <row r="49" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A49" s="2" t="s">
         <v>1205</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="2" t="s">
         <v>1205</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A50" t="s">
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+    </row>
+    <row r="50" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A50" s="2" t="s">
         <v>1206</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="2" t="s">
         <v>1206</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A51" t="s">
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+    </row>
+    <row r="51" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A51" s="2" t="s">
         <v>987</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="2" t="s">
         <v>987</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A52" t="s">
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+    </row>
+    <row r="52" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A52" s="2" t="s">
         <v>1048</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="2" t="s">
         <v>1048</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A53" t="s">
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+    </row>
+    <row r="53" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A53" s="2" t="s">
         <v>1049</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="2" t="s">
         <v>1049</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A54" t="s">
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+    </row>
+    <row r="54" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A54" s="2" t="s">
         <v>1120</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="2" t="s">
         <v>1120</v>
       </c>
-    </row>
-    <row r="55" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A55" t="s">
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+    </row>
+    <row r="55" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A55" s="2" t="s">
         <v>1121</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="2" t="s">
         <v>1121</v>
       </c>
-    </row>
-    <row r="56" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A56" t="s">
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+    </row>
+    <row r="56" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A56" s="2" t="s">
         <v>1122</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="2" t="s">
         <v>1122</v>
       </c>
-    </row>
-    <row r="57" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A57" t="s">
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+    </row>
+    <row r="57" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A57" s="2" t="s">
         <v>1202</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="2" t="s">
         <v>1202</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A58" s="8" t="s">
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+    </row>
+    <row r="58" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A58" s="9" t="s">
         <v>1207</v>
       </c>
-      <c r="B58" s="8" t="s">
+      <c r="B58" s="9" t="s">
         <v>1207</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A59" t="s">
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+    </row>
+    <row r="59" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A59" s="2" t="s">
         <v>1209</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="2" t="s">
         <v>1209</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="62" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="63" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="64" spans="1:2" ht="14.25" customHeight="1"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+    </row>
+    <row r="60" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>1210</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>1210</v>
+      </c>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+    </row>
+    <row r="61" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="62" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="63" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="64" spans="1:4" ht="14.25" customHeight="1"/>
     <row r="65" ht="14.25" customHeight="1"/>
     <row r="66" ht="14.25" customHeight="1"/>
     <row r="67" ht="14.25" customHeight="1"/>
@@ -9228,45 +9364,45 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>195</v>
+        <v>494</v>
       </c>
       <c r="B70" t="s">
-        <v>669</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B71" t="s">
-        <v>670</v>
-      </c>
-      <c r="C71" t="s">
-        <v>522</v>
+        <v>669</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>513</v>
+        <v>196</v>
       </c>
       <c r="B72" t="s">
-        <v>671</v>
+        <v>670</v>
+      </c>
+      <c r="C72" t="s">
+        <v>522</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>487</v>
+        <v>513</v>
       </c>
       <c r="B73" t="s">
-        <v>488</v>
+        <v>671</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="B74" t="s">
-        <v>1096</v>
+        <v>488</v>
       </c>
     </row>
     <row r="75" spans="1:3">

</xml_diff>

<commit_message>
added CQ workflow for AZ
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F0857E-F12D-4A46-AE7D-A85A54D746FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED3CEBC6-4E14-4B1F-8367-2E21DE97E982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1516" uniqueCount="1211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1698" uniqueCount="1393">
   <si>
     <t>Name</t>
   </si>
@@ -3676,6 +3676,552 @@
   </si>
   <si>
     <t>TX_NoAssetsCheckProperties</t>
+  </si>
+  <si>
+    <t>The Certification Questionnaire is missing for one or more adult household members. </t>
+  </si>
+  <si>
+    <t>Name has not been completed on the Certification Questionnaire. </t>
+  </si>
+  <si>
+    <t>Unit Number has not been completed on the Certification Questionnaire. </t>
+  </si>
+  <si>
+    <t>Property Name has not been completed on the Certification Questionnaire. </t>
+  </si>
+  <si>
+    <t>One of the Move-In, Recertification, or Addition of Household checkboxes has not been selected. </t>
+  </si>
+  <si>
+    <t>Question 1 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 1 has been answered Yes, but the PHA Name has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 1 has been answered Yes. Upload HAP contract with final signed documents. </t>
+  </si>
+  <si>
+    <t>Question 2 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 2 has been answered Yes, but the Program Name and/or the Organization Providing Rental Assistance has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 3 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 3 has been answered Yes, but the required income information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 4 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 4 has been answered Yes, but the required income information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 5 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 5 has been answered Yes, but the required income information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 6 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 6 has been answered Yes, but Monthly Gross Income has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 7 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 7 has been answered Yes, but Monthly Gross Income has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 8 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 8 has been answered Yes, but Monthly Gross Income has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 9 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 9 has been answered Yes, but the required income information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 9 has been answered Yes, but one or more household member names listed in the income section does not match the ICW. </t>
+  </si>
+  <si>
+    <t>Question 10 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 10 has been answered Yes, but Monthly Gross Income has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 11 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 11 has been answered Yes, but Monthly Gross Income has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 12 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 12 has been answered Yes, but Monthly Gross Income has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 13 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 13 has not been fully completed. </t>
+  </si>
+  <si>
+    <t>Question 14 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 14 has been answered Yes, but Monthly Gross Income has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 15 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 15 has been answered Yes, but the required income information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 16 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 16 has been answered Yes, but Monthly Net Income has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 17 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 17 has been answered Yes, but Amount Per Semester has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 18 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 19 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>One or more income types documented on the Certification Questionnaire do not match the income information listed on the ICW. </t>
+  </si>
+  <si>
+    <t>Question 20 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 20 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 21 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 21 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 22 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 22 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 23 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 23 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 24 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 24 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 25 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 25 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 26 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 26 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 27 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 27 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 28 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 28 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 29 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 29 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 30 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 30 has been answered Yes, but Cash Value has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 31 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 31 has been answered Yes, but Cash Value has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 32 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 32 has been answered Yes. Manual review is needed. </t>
+  </si>
+  <si>
+    <t>Question 33 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 33 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 34 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 34 has been answered Yes, but Current Balance has not been provided. </t>
+  </si>
+  <si>
+    <t>Question 35 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 35 has been answered Yes, but the required asset information has not been completed. </t>
+  </si>
+  <si>
+    <t>Question 36 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 36 has been answered Yes, but Amount Received has not been provided. </t>
+  </si>
+  <si>
+    <t>One or more asset type(s), source(s), and/or cash value(s) documented on the Certification Questionnaire do not match the asset information listed on the ICW. </t>
+  </si>
+  <si>
+    <t>Question 37 has not been answered Yes or No. </t>
+  </si>
+  <si>
+    <t>Question 37 has been answered No, but one or more of Questions 38–54 have been completed. </t>
+  </si>
+  <si>
+    <t>Question 37 has been answered Yes, but the required student certification questions have not been completed. </t>
+  </si>
+  <si>
+    <t>Question 39 has been answered Yes, but the required questions have not been completed. </t>
+  </si>
+  <si>
+    <t>Application is for a HOME/SHTF unit, but Questions 45–50 have not been fully completed. </t>
+  </si>
+  <si>
+    <t>Questions 51–54 have not been completed. </t>
+  </si>
+  <si>
+    <t>Certification Questionnaire has not been signed. </t>
+  </si>
+  <si>
+    <t>Printed Name has not been completed on the Certification Questionnaire. </t>
+  </si>
+  <si>
+    <t>Certification Questionnaire has not been dated. </t>
+  </si>
+  <si>
+    <t>Date listed on the Certification Questionnaire is not within 120 days of Move-In date. </t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Certification Questionnaire. Manual review is needed. </t>
+  </si>
+  <si>
+    <t>CQExists</t>
+  </si>
+  <si>
+    <t>CQ_Name</t>
+  </si>
+  <si>
+    <t>CQ_UnitNumber</t>
+  </si>
+  <si>
+    <t>CQ_PropertyName</t>
+  </si>
+  <si>
+    <t>CQ_Checkboxes</t>
+  </si>
+  <si>
+    <t>CQ_Q1Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q1YesNoPHAName</t>
+  </si>
+  <si>
+    <t>CQ_Q2YesNoProgramName</t>
+  </si>
+  <si>
+    <t>CQ_Q3NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q5NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q6NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q7NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q8NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q9NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q10NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q2NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q1NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q4NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q3Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q4Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q5Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q6Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q7Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q8Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q9Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q10Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q9YesNoICWNamesMatch</t>
+  </si>
+  <si>
+    <t>CQ_Q11NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q11Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q19NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q18NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q17Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q17NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q12NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q12Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q13NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q13Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q14NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q14Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q15NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q15Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q16NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q16Yes</t>
+  </si>
+  <si>
+    <t>CQ_IncomeType</t>
+  </si>
+  <si>
+    <t>CQ_Q20NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q20Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q30NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q31NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q32NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q33NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q34NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q35NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q36NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q37NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q30Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q31Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q34Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q21NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q21Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q22NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q22Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q23NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q23Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q24NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q24Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q25Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q25NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q26NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q26Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q27NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q27Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q28NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q28Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q29NotYesNo</t>
+  </si>
+  <si>
+    <t>CQ_Q29Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q32Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q37Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q39Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q33Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q35Yes</t>
+  </si>
+  <si>
+    <t>CQ_Q36Yes</t>
+  </si>
+  <si>
+    <t>CQ_AssetType</t>
+  </si>
+  <si>
+    <t>CQ_Q37No</t>
+  </si>
+  <si>
+    <t>CQ_HomeSHTF</t>
+  </si>
+  <si>
+    <t>CQ_Q51-54NotCompleted</t>
+  </si>
+  <si>
+    <t>CQ_NotSigned</t>
+  </si>
+  <si>
+    <t>CQ_PrintedName</t>
+  </si>
+  <si>
+    <t>CQ_NotDated</t>
+  </si>
+  <si>
+    <t>CQ_CheckMoveInDate</t>
+  </si>
+  <si>
+    <t>CQ_FindingError</t>
+  </si>
+  <si>
+    <t>CQ</t>
+  </si>
+  <si>
+    <t>Certification Questionnaire</t>
   </si>
 </sst>
 </file>
@@ -4611,7 +5157,14 @@
         <v>989</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="61" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A61" t="s">
+        <v>1391</v>
+      </c>
+      <c r="B61" t="s">
+        <v>1392</v>
+      </c>
+    </row>
     <row r="62" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="63" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="64" spans="1:3" ht="14.25" customHeight="1"/>
@@ -8780,7 +9333,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C525"/>
+  <dimension ref="A1:C616"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" bestFit="1" customWidth="1"/>
@@ -13134,6 +13687,726 @@
         <v>1127</v>
       </c>
     </row>
+    <row r="527" spans="1:3">
+      <c r="A527" t="s">
+        <v>1301</v>
+      </c>
+      <c r="B527" t="s">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="528" spans="1:3">
+      <c r="A528" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B528" t="s">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="529" spans="1:2">
+      <c r="A529" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B529" t="s">
+        <v>1213</v>
+      </c>
+    </row>
+    <row r="530" spans="1:2">
+      <c r="A530" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B530" t="s">
+        <v>1214</v>
+      </c>
+    </row>
+    <row r="531" spans="1:2">
+      <c r="A531" t="s">
+        <v>1305</v>
+      </c>
+      <c r="B531" t="s">
+        <v>1215</v>
+      </c>
+    </row>
+    <row r="532" spans="1:2">
+      <c r="A532" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B532" t="s">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="533" spans="1:2">
+      <c r="A533" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B533" t="s">
+        <v>1217</v>
+      </c>
+    </row>
+    <row r="534" spans="1:2">
+      <c r="A534" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B534" t="s">
+        <v>1218</v>
+      </c>
+    </row>
+    <row r="535" spans="1:2">
+      <c r="A535" t="s">
+        <v>1316</v>
+      </c>
+      <c r="B535" t="s">
+        <v>1219</v>
+      </c>
+    </row>
+    <row r="536" spans="1:2">
+      <c r="A536" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B536" t="s">
+        <v>1220</v>
+      </c>
+    </row>
+    <row r="537" spans="1:2">
+      <c r="A537" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B537" t="s">
+        <v>1221</v>
+      </c>
+    </row>
+    <row r="538" spans="1:2">
+      <c r="A538" t="s">
+        <v>1319</v>
+      </c>
+      <c r="B538" t="s">
+        <v>1222</v>
+      </c>
+    </row>
+    <row r="539" spans="1:2">
+      <c r="A539" t="s">
+        <v>1318</v>
+      </c>
+      <c r="B539" t="s">
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="540" spans="1:2">
+      <c r="A540" t="s">
+        <v>1320</v>
+      </c>
+      <c r="B540" t="s">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="541" spans="1:2">
+      <c r="A541" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B541" t="s">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="542" spans="1:2">
+      <c r="A542" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B542" t="s">
+        <v>1226</v>
+      </c>
+    </row>
+    <row r="543" spans="1:2">
+      <c r="A543" t="s">
+        <v>1311</v>
+      </c>
+      <c r="B543" t="s">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="544" spans="1:2">
+      <c r="A544" t="s">
+        <v>1322</v>
+      </c>
+      <c r="B544" t="s">
+        <v>1228</v>
+      </c>
+    </row>
+    <row r="545" spans="1:2">
+      <c r="A545" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B545" t="s">
+        <v>1229</v>
+      </c>
+    </row>
+    <row r="546" spans="1:2">
+      <c r="A546" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B546" t="s">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="547" spans="1:2">
+      <c r="A547" t="s">
+        <v>1313</v>
+      </c>
+      <c r="B547" t="s">
+        <v>1231</v>
+      </c>
+    </row>
+    <row r="548" spans="1:2">
+      <c r="A548" t="s">
+        <v>1324</v>
+      </c>
+      <c r="B548" t="s">
+        <v>1232</v>
+      </c>
+    </row>
+    <row r="549" spans="1:2">
+      <c r="A549" t="s">
+        <v>1314</v>
+      </c>
+      <c r="B549" t="s">
+        <v>1233</v>
+      </c>
+    </row>
+    <row r="550" spans="1:2">
+      <c r="A550" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B550" t="s">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="551" spans="1:2">
+      <c r="A551" t="s">
+        <v>1327</v>
+      </c>
+      <c r="B551" t="s">
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="552" spans="1:2">
+      <c r="A552" t="s">
+        <v>1315</v>
+      </c>
+      <c r="B552" t="s">
+        <v>1236</v>
+      </c>
+    </row>
+    <row r="553" spans="1:2">
+      <c r="A553" t="s">
+        <v>1326</v>
+      </c>
+      <c r="B553" t="s">
+        <v>1237</v>
+      </c>
+    </row>
+    <row r="554" spans="1:2">
+      <c r="A554" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B554" t="s">
+        <v>1238</v>
+      </c>
+    </row>
+    <row r="555" spans="1:2">
+      <c r="A555" t="s">
+        <v>1329</v>
+      </c>
+      <c r="B555" t="s">
+        <v>1239</v>
+      </c>
+    </row>
+    <row r="556" spans="1:2">
+      <c r="A556" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B556" t="s">
+        <v>1240</v>
+      </c>
+    </row>
+    <row r="557" spans="1:2">
+      <c r="A557" t="s">
+        <v>1335</v>
+      </c>
+      <c r="B557" t="s">
+        <v>1241</v>
+      </c>
+    </row>
+    <row r="558" spans="1:2">
+      <c r="A558" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B558" t="s">
+        <v>1242</v>
+      </c>
+    </row>
+    <row r="559" spans="1:2">
+      <c r="A559" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B559" t="s">
+        <v>1243</v>
+      </c>
+    </row>
+    <row r="560" spans="1:2">
+      <c r="A560" t="s">
+        <v>1338</v>
+      </c>
+      <c r="B560" t="s">
+        <v>1244</v>
+      </c>
+    </row>
+    <row r="561" spans="1:2">
+      <c r="A561" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B561" t="s">
+        <v>1245</v>
+      </c>
+    </row>
+    <row r="562" spans="1:2">
+      <c r="A562" t="s">
+        <v>1340</v>
+      </c>
+      <c r="B562" t="s">
+        <v>1246</v>
+      </c>
+    </row>
+    <row r="563" spans="1:2">
+      <c r="A563" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B563" t="s">
+        <v>1247</v>
+      </c>
+    </row>
+    <row r="564" spans="1:2">
+      <c r="A564" t="s">
+        <v>1342</v>
+      </c>
+      <c r="B564" t="s">
+        <v>1248</v>
+      </c>
+    </row>
+    <row r="565" spans="1:2">
+      <c r="A565" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B565" t="s">
+        <v>1249</v>
+      </c>
+    </row>
+    <row r="566" spans="1:2">
+      <c r="A566" t="s">
+        <v>1333</v>
+      </c>
+      <c r="B566" t="s">
+        <v>1250</v>
+      </c>
+    </row>
+    <row r="567" spans="1:2">
+      <c r="A567" t="s">
+        <v>1332</v>
+      </c>
+      <c r="B567" t="s">
+        <v>1251</v>
+      </c>
+    </row>
+    <row r="568" spans="1:2">
+      <c r="A568" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B568" t="s">
+        <v>1252</v>
+      </c>
+    </row>
+    <row r="569" spans="1:2">
+      <c r="A569" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B569" t="s">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="570" spans="1:2">
+      <c r="A570" t="s">
+        <v>1344</v>
+      </c>
+      <c r="B570" t="s">
+        <v>1254</v>
+      </c>
+    </row>
+    <row r="571" spans="1:2">
+      <c r="A571" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B571" t="s">
+        <v>1255</v>
+      </c>
+    </row>
+    <row r="572" spans="1:2">
+      <c r="A572" t="s">
+        <v>1346</v>
+      </c>
+      <c r="B572" t="s">
+        <v>1256</v>
+      </c>
+    </row>
+    <row r="573" spans="1:2">
+      <c r="A573" t="s">
+        <v>1358</v>
+      </c>
+      <c r="B573" t="s">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="574" spans="1:2">
+      <c r="A574" t="s">
+        <v>1359</v>
+      </c>
+      <c r="B574" t="s">
+        <v>1258</v>
+      </c>
+    </row>
+    <row r="575" spans="1:2">
+      <c r="A575" t="s">
+        <v>1360</v>
+      </c>
+      <c r="B575" t="s">
+        <v>1259</v>
+      </c>
+    </row>
+    <row r="576" spans="1:2">
+      <c r="A576" t="s">
+        <v>1361</v>
+      </c>
+      <c r="B576" t="s">
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="577" spans="1:2">
+      <c r="A577" t="s">
+        <v>1362</v>
+      </c>
+      <c r="B577" t="s">
+        <v>1261</v>
+      </c>
+    </row>
+    <row r="578" spans="1:2">
+      <c r="A578" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B578" t="s">
+        <v>1262</v>
+      </c>
+    </row>
+    <row r="579" spans="1:2">
+      <c r="A579" t="s">
+        <v>1364</v>
+      </c>
+      <c r="B579" t="s">
+        <v>1263</v>
+      </c>
+    </row>
+    <row r="580" spans="1:2">
+      <c r="A580" t="s">
+        <v>1365</v>
+      </c>
+      <c r="B580" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="581" spans="1:2">
+      <c r="A581" t="s">
+        <v>1367</v>
+      </c>
+      <c r="B581" t="s">
+        <v>1265</v>
+      </c>
+    </row>
+    <row r="582" spans="1:2">
+      <c r="A582" t="s">
+        <v>1366</v>
+      </c>
+      <c r="B582" t="s">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="583" spans="1:2">
+      <c r="A583" t="s">
+        <v>1368</v>
+      </c>
+      <c r="B583" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="584" spans="1:2">
+      <c r="A584" t="s">
+        <v>1369</v>
+      </c>
+      <c r="B584" t="s">
+        <v>1268</v>
+      </c>
+    </row>
+    <row r="585" spans="1:2">
+      <c r="A585" t="s">
+        <v>1370</v>
+      </c>
+      <c r="B585" t="s">
+        <v>1269</v>
+      </c>
+    </row>
+    <row r="586" spans="1:2">
+      <c r="A586" t="s">
+        <v>1371</v>
+      </c>
+      <c r="B586" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="587" spans="1:2">
+      <c r="A587" t="s">
+        <v>1372</v>
+      </c>
+      <c r="B587" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="588" spans="1:2">
+      <c r="A588" t="s">
+        <v>1373</v>
+      </c>
+      <c r="B588" t="s">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="589" spans="1:2">
+      <c r="A589" t="s">
+        <v>1374</v>
+      </c>
+      <c r="B589" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="590" spans="1:2">
+      <c r="A590" t="s">
+        <v>1375</v>
+      </c>
+      <c r="B590" t="s">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="591" spans="1:2">
+      <c r="A591" t="s">
+        <v>1347</v>
+      </c>
+      <c r="B591" t="s">
+        <v>1275</v>
+      </c>
+    </row>
+    <row r="592" spans="1:2">
+      <c r="A592" t="s">
+        <v>1355</v>
+      </c>
+      <c r="B592" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="593" spans="1:2">
+      <c r="A593" t="s">
+        <v>1348</v>
+      </c>
+      <c r="B593" t="s">
+        <v>1277</v>
+      </c>
+    </row>
+    <row r="594" spans="1:2">
+      <c r="A594" t="s">
+        <v>1356</v>
+      </c>
+      <c r="B594" t="s">
+        <v>1278</v>
+      </c>
+    </row>
+    <row r="595" spans="1:2">
+      <c r="A595" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B595" t="s">
+        <v>1279</v>
+      </c>
+    </row>
+    <row r="596" spans="1:2">
+      <c r="A596" t="s">
+        <v>1376</v>
+      </c>
+      <c r="B596" t="s">
+        <v>1280</v>
+      </c>
+    </row>
+    <row r="597" spans="1:2">
+      <c r="A597" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B597" t="s">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="598" spans="1:2">
+      <c r="A598" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B598" t="s">
+        <v>1282</v>
+      </c>
+    </row>
+    <row r="599" spans="1:2">
+      <c r="A599" t="s">
+        <v>1351</v>
+      </c>
+      <c r="B599" t="s">
+        <v>1283</v>
+      </c>
+    </row>
+    <row r="600" spans="1:2">
+      <c r="A600" t="s">
+        <v>1357</v>
+      </c>
+      <c r="B600" t="s">
+        <v>1284</v>
+      </c>
+    </row>
+    <row r="601" spans="1:2">
+      <c r="A601" t="s">
+        <v>1352</v>
+      </c>
+      <c r="B601" t="s">
+        <v>1285</v>
+      </c>
+    </row>
+    <row r="602" spans="1:2">
+      <c r="A602" t="s">
+        <v>1380</v>
+      </c>
+      <c r="B602" t="s">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="603" spans="1:2">
+      <c r="A603" t="s">
+        <v>1353</v>
+      </c>
+      <c r="B603" t="s">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="604" spans="1:2">
+      <c r="A604" t="s">
+        <v>1381</v>
+      </c>
+      <c r="B604" t="s">
+        <v>1288</v>
+      </c>
+    </row>
+    <row r="605" spans="1:2">
+      <c r="A605" t="s">
+        <v>1382</v>
+      </c>
+      <c r="B605" t="s">
+        <v>1289</v>
+      </c>
+    </row>
+    <row r="606" spans="1:2">
+      <c r="A606" t="s">
+        <v>1354</v>
+      </c>
+      <c r="B606" t="s">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="607" spans="1:2">
+      <c r="A607" t="s">
+        <v>1383</v>
+      </c>
+      <c r="B607" t="s">
+        <v>1291</v>
+      </c>
+    </row>
+    <row r="608" spans="1:2">
+      <c r="A608" t="s">
+        <v>1377</v>
+      </c>
+      <c r="B608" t="s">
+        <v>1292</v>
+      </c>
+    </row>
+    <row r="609" spans="1:2">
+      <c r="A609" t="s">
+        <v>1378</v>
+      </c>
+      <c r="B609" t="s">
+        <v>1293</v>
+      </c>
+    </row>
+    <row r="610" spans="1:2">
+      <c r="A610" t="s">
+        <v>1384</v>
+      </c>
+      <c r="B610" t="s">
+        <v>1294</v>
+      </c>
+    </row>
+    <row r="611" spans="1:2">
+      <c r="A611" t="s">
+        <v>1385</v>
+      </c>
+      <c r="B611" t="s">
+        <v>1295</v>
+      </c>
+    </row>
+    <row r="612" spans="1:2">
+      <c r="A612" t="s">
+        <v>1386</v>
+      </c>
+      <c r="B612" t="s">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="613" spans="1:2">
+      <c r="A613" t="s">
+        <v>1387</v>
+      </c>
+      <c r="B613" t="s">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="614" spans="1:2">
+      <c r="A614" t="s">
+        <v>1388</v>
+      </c>
+      <c r="B614" t="s">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="615" spans="1:2">
+      <c r="A615" t="s">
+        <v>1389</v>
+      </c>
+      <c r="B615" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="616" spans="1:2">
+      <c r="A616" t="s">
+        <v>1390</v>
+      </c>
+      <c r="B616" t="s">
+        <v>1300</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C525" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}"/>
   <conditionalFormatting sqref="A479:A481 A476:A477 A461:A471 A473:A474">

</xml_diff>

<commit_message>
raluca's changes for CQ document
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bagi.Elangovan\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2694CD-A8D0-4D31-B03F-86DCBAFAD7B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D90B2D51-22DA-4A6A-891E-782A3E845F86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -4233,7 +4233,7 @@
     <t>Updated by Harman</t>
   </si>
   <si>
-    <t>C:\Users\Bagi.Elangovan\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
bagi s changes and changes to SSBL workflow from my side
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\1028\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5571271E-9C6D-4B6F-A536-0A645DE5B364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{059DD523-6F96-4FA2-B934-F7A3DBD700F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22560" windowHeight="11655" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2280" uniqueCount="1402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2282" uniqueCount="1403">
   <si>
     <t>Name</t>
   </si>
@@ -4249,6 +4249,9 @@
   </si>
   <si>
     <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>COLACalcDate</t>
   </si>
 </sst>
 </file>
@@ -8384,7 +8387,14 @@
       <c r="C59" s="2"/>
       <c r="D59" s="2"/>
     </row>
-    <row r="60" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="60" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>1402</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>1402</v>
+      </c>
+    </row>
     <row r="61" spans="1:4" ht="14.25" customHeight="1"/>
     <row r="62" spans="1:4" ht="14.25" customHeight="1"/>
     <row r="63" spans="1:4" ht="14.25" customHeight="1"/>

</xml_diff>